<commit_message>
Checkpoint: Series Seed sheet built
</commit_message>
<xml_diff>
--- a/runs/20260414-171016/models/model.xlsx
+++ b/runs/20260414-171016/models/model.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B7FAD96-C548-FB4A-BCC9-2853A08B12EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD2B83F2-323E-6540-98D9-2E66D7A9DD26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Series A" sheetId="136" r:id="rId1"/>
-    <sheet name="Detailed Cap Table" sheetId="138" r:id="rId2"/>
-    <sheet name="SAFE Investments" sheetId="139" r:id="rId3"/>
+    <sheet name="Detailed Cap Table" sheetId="138" r:id="rId1"/>
+    <sheet name="SAFE Investments" sheetId="139" r:id="rId2"/>
+    <sheet name="Series Seed" sheetId="140" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>Total</t>
   </si>
@@ -193,15 +193,15 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t>SAFE Investments</t>
+  </si>
+  <si>
     <t xml:space="preserve">Common </t>
   </si>
   <si>
     <t xml:space="preserve">Option </t>
   </si>
   <si>
-    <t>Series A</t>
-  </si>
-  <si>
     <t>Total Capitalization</t>
   </si>
   <si>
@@ -211,24 +211,21 @@
     <t>$</t>
   </si>
   <si>
-    <t>Preferred</t>
-  </si>
-  <si>
     <t>Pool +</t>
   </si>
   <si>
     <t>Total FD</t>
   </si>
   <si>
+    <t>%</t>
+  </si>
+  <si>
     <t>Shares</t>
   </si>
   <si>
     <t xml:space="preserve"> Invested</t>
   </si>
   <si>
-    <t>Pre-SAFE</t>
-  </si>
-  <si>
     <t>Pre A</t>
   </si>
   <si>
@@ -241,84 +238,40 @@
     <t>Total Common</t>
   </si>
   <si>
-    <t>Other Series A Investors</t>
-  </si>
-  <si>
     <t>Totals</t>
   </si>
   <si>
-    <t>Price per Share</t>
-  </si>
-  <si>
-    <t>Pre-Money Valuation</t>
-  </si>
-  <si>
-    <t>Post-Money Valuation</t>
-  </si>
-  <si>
-    <t>Series A Assumptions:</t>
-  </si>
-  <si>
-    <t>Total Raised</t>
-  </si>
-  <si>
-    <t>Pre-Money Valuation Step-up</t>
-  </si>
-  <si>
     <t>Other Common Shareholders</t>
   </si>
   <si>
     <t>ESOP Issued &amp; Outstanding</t>
   </si>
   <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
     <t>Other SAFE Investors</t>
   </si>
   <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
   </si>
   <si>
-    <t xml:space="preserve">% </t>
-  </si>
-  <si>
-    <t>1011 VENTURES SERIES A</t>
+    <t>SIDEKICK (THINK MORE SECURITY) &amp; 1011 SERIES SEED</t>
   </si>
   <si>
     <t>SAFE Valuation Cap</t>
-  </si>
-  <si>
-    <t>SIDEKICK (THINK MORE SECURITY)</t>
-  </si>
-  <si>
-    <t>SAFE Conv</t>
-  </si>
-  <si>
-    <t>ESOP Available / Pool Expansion</t>
-  </si>
-  <si>
-    <t>Preferred Rounds:</t>
-  </si>
-  <si>
-    <t>% Ownership (New Money)</t>
-  </si>
-  <si>
-    <t>Option Pool Expansion %</t>
-  </si>
-  <si>
-    <t>SAFE Conversion Price</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0_-;_-[$$-409]* \(#,##0\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="0.0%_);\(0.0%\);0.0%_);@_)"/>
-    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.0000_-;_-[$$-409]* \(#,##0.0000\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -455,19 +408,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Garamond"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Garamond"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Garamond"/>
       <family val="1"/>
@@ -479,9 +419,8 @@
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Garamond"/>
       <family val="1"/>
     </font>
@@ -505,6 +444,13 @@
       <name val="Garamond"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -687,7 +633,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -892,6 +838,19 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -997,133 +956,112 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="37" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="37" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="37" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="37" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="37" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="20" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="20" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="37" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="37" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="19" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1518,653 +1456,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{343D6CA6-81A9-1E49-B4DF-137DA23E3554}">
-  <dimension ref="B1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="6.33203125" customWidth="1"/>
-    <col min="2" max="2" width="35.5" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="0.5" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" customWidth="1"/>
-    <col min="8" max="8" width="0.5" customWidth="1"/>
-    <col min="9" max="9" width="15.5" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="0.5" customWidth="1"/>
-    <col min="12" max="12" width="13.83203125" customWidth="1"/>
-    <col min="13" max="13" width="0.5" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
-    <col min="15" max="15" width="9.33203125" customWidth="1"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1"/>
-    <col min="17" max="17" width="15.5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B1" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-    </row>
-    <row r="2" spans="2:17" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-    </row>
-    <row r="3" spans="2:17" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-    </row>
-    <row r="4" spans="2:17" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="20"/>
-      <c r="G4" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="J4" s="25"/>
-      <c r="L4" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="N4" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="O4" s="25"/>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="C5" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="G5" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="I5" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="J5" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="L5" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="N5" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="O5" s="25" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="E6" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="I6" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="J6" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="L6" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="N6" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="O6" s="37" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B7" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="35"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="35"/>
-      <c r="O7" s="50"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B8" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="9" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D8" s="49"/>
-      <c r="E8" s="6"/>
-      <c r="G8" s="11"/>
-      <c r="I8" s="49"/>
-      <c r="J8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="N8" s="6" t="e">
-        <f>C8+E8+G8+J8+L8</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O8" s="18" t="e">
-        <f>N8/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B9" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="9" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D9" s="49"/>
-      <c r="E9" s="6"/>
-      <c r="G9" s="11"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="N9" s="6" t="e">
-        <f>C9+E9+G9+J9+L9</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O9" s="18" t="e">
-        <f>N9/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B10" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="9" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D10" s="49"/>
-      <c r="E10" s="6"/>
-      <c r="G10" s="11"/>
-      <c r="I10" s="49"/>
-      <c r="J10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="N10" s="6" t="e">
-        <f>C10+E10+G10+J10+L10</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O10" s="18" t="e">
-        <f>N10/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B11" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="49"/>
-      <c r="E11" s="6"/>
-      <c r="G11" s="9" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I11" s="49"/>
-      <c r="J11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="N11" s="6" t="e">
-        <f>C11+E11+G11+J11+L11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O11" s="18" t="e">
-        <f>N11/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B12" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="6"/>
-      <c r="G12" s="9" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I12" s="49"/>
-      <c r="J12" s="6"/>
-      <c r="L12" s="6">
-        <f>IFERROR(ROUND(0.1*N21-G12,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="N12" s="6" t="e">
-        <f>C12+E12+G12+J12+L12</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O12" s="18" t="e">
-        <f>N12/$N$21</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Q12" s="1">
-        <f>IFERROR((G12+L12)/N21,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="15"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="6"/>
-      <c r="G13" s="11"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="18"/>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B14" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="44" t="e">
-        <f>SUM(C8:C12)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D14" s="41"/>
-      <c r="E14" s="40">
-        <f>SUM(E8:E12)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="44" t="e">
-        <f>SUM(G8:G12)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I14" s="41"/>
-      <c r="J14" s="40">
-        <f>SUM(J8:J12)</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="44">
-        <f>SUM(L8:L12)</f>
-        <v>0</v>
-      </c>
-      <c r="N14" s="44" t="e">
-        <f>SUM(N8:N12)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O14" s="45" t="e">
-        <f>N14/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B15" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="6"/>
-      <c r="G15" s="11"/>
-      <c r="I15" s="49"/>
-      <c r="J15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="18"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B16" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="10" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E16" s="6">
-        <f ca="1">IFERROR(ROUND(D16/$E$23,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="11"/>
-      <c r="I16" s="7">
-        <v>5000000</v>
-      </c>
-      <c r="J16" s="6">
-        <f ca="1">IFERROR(ROUND(I16/$J$23,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="6"/>
-      <c r="N16" s="6">
-        <f ca="1">C16+E16+G16+J16+L16</f>
-        <v>0</v>
-      </c>
-      <c r="O16" s="18" t="e">
-        <f ca="1">N16/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B17" s="15">
-        <v>1011</v>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="6"/>
-      <c r="G17" s="11"/>
-      <c r="I17" s="7">
-        <v>12000000</v>
-      </c>
-      <c r="J17" s="6">
-        <f ca="1">IFERROR(ROUND(I17/$J$23,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L17" s="6"/>
-      <c r="N17" s="6">
-        <f ca="1">C17+E17+G17+J17+L17</f>
-        <v>0</v>
-      </c>
-      <c r="O17" s="18" t="e">
-        <f ca="1">N17/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B18" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="49"/>
-      <c r="E18" s="6"/>
-      <c r="G18" s="11"/>
-      <c r="I18" s="7">
-        <v>3000000</v>
-      </c>
-      <c r="J18" s="6">
-        <f ca="1">IFERROR(ROUND(I18/$J$23,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L18" s="6"/>
-      <c r="N18" s="6">
-        <f ca="1">C18+E18+G18+J18+L18</f>
-        <v>0</v>
-      </c>
-      <c r="O18" s="18" t="e">
-        <f ca="1">N18/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B19" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="10" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E19" s="6">
-        <f ca="1">IFERROR(ROUND(D19/$E$23,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G19" s="11"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="N19" s="6">
-        <f ca="1">C19+E19+G19+J19+L19</f>
-        <v>0</v>
-      </c>
-      <c r="O19" s="18" t="e">
-        <f ca="1">N19/$N$21</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B20" s="16"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="49"/>
-      <c r="E20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="I20" s="49"/>
-      <c r="J20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="42"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B21" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" s="44" t="e">
-        <f>SUM(C8:C19)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D21" s="47" t="e">
-        <f>SUM(D8:D19)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E21" s="46">
-        <f ca="1">SUM(E8:E19)</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="44" t="e">
-        <f>SUM(G8:G19)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I21" s="47">
-        <f>SUM(I8:I19)</f>
-        <v>20000000</v>
-      </c>
-      <c r="J21" s="46">
-        <f ca="1">SUM(J8:J19)</f>
-        <v>0</v>
-      </c>
-      <c r="L21" s="44">
-        <f>SUM(L8:L19)</f>
-        <v>0</v>
-      </c>
-      <c r="N21" s="44" t="e">
-        <f>SUM(N14,N16:N19)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O21" s="45" t="e">
-        <f>SUM(O14,O16:O19)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="22" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="16"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="G22" s="34"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="L22" s="34"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="51"/>
-    </row>
-    <row r="23" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="52">
-        <f ca="1">IFERROR(ROUND(50000000/(C14+G11+G12+E21),4),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="52">
-        <f ca="1">IFERROR(ROUND(J24/(C14+G11+G12+L12+E21),4),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="43"/>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B24" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="7">
-        <v>60000000</v>
-      </c>
-      <c r="L24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="43"/>
-    </row>
-    <row r="25" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="36"/>
-      <c r="J25" s="53">
-        <f>J24+I21</f>
-        <v>80000000</v>
-      </c>
-      <c r="K25" s="14"/>
-      <c r="L25" s="36"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="36"/>
-      <c r="O25" s="48"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B27" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B29" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="3"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B30" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" s="22">
-        <f>I21</f>
-        <v>20000000</v>
-      </c>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B31" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="C31" s="4">
-        <f>I21/J25</f>
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B32" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C32" s="8">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B33" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C33" s="39">
-        <v>50000000</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B34" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C34" s="21">
-        <f ca="1">E23</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3467316-53BC-114B-A078-C25AAB6A57B9}">
   <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2182,502 +1473,502 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="27"/>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="A1" s="8"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="28" t="s">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="27"/>
-      <c r="B3" s="28" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="F3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="27"/>
-      <c r="B4" s="27" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="29">
+      <c r="C4" s="10">
         <v>3600000</v>
       </c>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29">
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="30">
+      <c r="H4" s="11">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="10">
         <v>3600000</v>
       </c>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29">
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="11">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="10">
         <v>222187</v>
       </c>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29">
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="30">
+      <c r="H6" s="11">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="10">
         <v>592500</v>
       </c>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29">
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="11">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="27"/>
-      <c r="B8" s="27" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="10">
         <v>592500</v>
       </c>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29">
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="30">
+      <c r="H8" s="11">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="27"/>
-      <c r="B9" s="27" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="10">
         <v>13500</v>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="10">
         <v>98900</v>
       </c>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29">
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="30">
+      <c r="H9" s="11">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="10">
         <v>9000</v>
       </c>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29">
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="30">
+      <c r="H10" s="11">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10">
         <v>95000</v>
       </c>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29">
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="30">
+      <c r="H11" s="11">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29">
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10">
         <v>25000</v>
       </c>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29">
+      <c r="F12" s="10"/>
+      <c r="G12" s="10">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="30">
+      <c r="H12" s="11">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="27"/>
-      <c r="B13" s="27" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29">
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10">
         <v>41562</v>
       </c>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29">
+      <c r="F13" s="10"/>
+      <c r="G13" s="10">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="30">
+      <c r="H13" s="11">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27" t="s">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29">
+      <c r="C14" s="10"/>
+      <c r="D14" s="10">
         <v>285000</v>
       </c>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29">
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="11">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27" t="s">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29">
+      <c r="C15" s="10"/>
+      <c r="D15" s="10">
         <v>50000</v>
       </c>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29">
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="11">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27" t="s">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10">
         <v>285000</v>
       </c>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29">
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="11">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="27"/>
-      <c r="B17" s="27" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29">
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10">
         <v>96186</v>
       </c>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29">
+      <c r="F17" s="10"/>
+      <c r="G17" s="10">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="11">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="27"/>
-      <c r="B18" s="27" t="s">
+      <c r="A18" s="8"/>
+      <c r="B18" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10">
         <v>48095</v>
       </c>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29">
+      <c r="F18" s="10"/>
+      <c r="G18" s="10">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="30">
+      <c r="H18" s="11">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27" t="s">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29">
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10">
         <v>12395</v>
       </c>
-      <c r="G19" s="29">
+      <c r="G19" s="10">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="30">
+      <c r="H19" s="11">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="27"/>
-      <c r="B20" s="27" t="s">
+      <c r="A20" s="8"/>
+      <c r="B20" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29">
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10">
         <v>8333</v>
       </c>
-      <c r="G20" s="29">
+      <c r="G20" s="10">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="30">
+      <c r="H20" s="11">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="27"/>
-      <c r="B21" s="27" t="s">
+      <c r="A21" s="8"/>
+      <c r="B21" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29">
+      <c r="C21" s="10"/>
+      <c r="D21" s="10">
         <v>65105</v>
       </c>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29">
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="11">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="27"/>
-      <c r="J21" s="27"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="27"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
     </row>
     <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="27"/>
-      <c r="B23" s="28" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="29">
+      <c r="C23" s="10">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="29">
+      <c r="D23" s="10">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="29">
+      <c r="E23" s="10">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="29">
+      <c r="F23" s="10">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="29">
+      <c r="G23" s="10">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="30"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A6BC71C-70E7-7F4D-8D3B-146049E1735A}">
   <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2691,341 +1982,660 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="27"/>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
+      <c r="A1" s="8"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="27"/>
-      <c r="B3" s="28" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="27"/>
-      <c r="E3" s="28" t="s">
+      <c r="D3" s="8"/>
+      <c r="E3" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="27"/>
+      <c r="F3" s="8"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="27"/>
-      <c r="B4" s="27" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="31">
+      <c r="C4" s="12">
         <v>25000</v>
       </c>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="27"/>
+      <c r="F4" s="8"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="12">
         <v>25000</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="12">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="12">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="27"/>
-      <c r="B8" s="27" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="12">
         <v>16566</v>
       </c>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="F8" s="27"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="27"/>
-      <c r="B9" s="27" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="12">
         <v>250000</v>
       </c>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="12">
         <v>100000</v>
       </c>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="12">
         <v>300000</v>
       </c>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27" t="s">
+      <c r="D11" s="8"/>
+      <c r="E11" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="27"/>
+      <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="12">
         <v>37500</v>
       </c>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27" t="s">
+      <c r="D12" s="8"/>
+      <c r="E12" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="27"/>
+      <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="27"/>
-      <c r="B13" s="27" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="12">
         <v>250000</v>
       </c>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27" t="s">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="12">
         <v>100000</v>
       </c>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27" t="s">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="12">
         <v>41164</v>
       </c>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="F15" s="27"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27" t="s">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="12">
         <v>2328778</v>
       </c>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="F16" s="27"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="27"/>
-      <c r="B17" s="27" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="31">
+      <c r="C17" s="12">
         <v>1506000</v>
       </c>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27" t="s">
+      <c r="D17" s="8"/>
+      <c r="E17" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="27"/>
+      <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="27"/>
-      <c r="B18" s="27" t="s">
+      <c r="A18" s="8"/>
+      <c r="B18" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="12">
         <v>50000</v>
       </c>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27" t="s">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="31">
+      <c r="C19" s="12">
         <v>212500</v>
       </c>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27" t="s">
+      <c r="D19" s="8"/>
+      <c r="E19" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="27"/>
+      <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="27"/>
-      <c r="B20" s="27" t="s">
+      <c r="A20" s="8"/>
+      <c r="B20" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="31">
+      <c r="C20" s="12">
         <v>25000</v>
       </c>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="27"/>
-      <c r="B21" s="27" t="s">
+      <c r="A21" s="8"/>
+      <c r="B21" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="31">
+      <c r="C21" s="12">
         <v>61746</v>
       </c>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="F21" s="27"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="27"/>
-      <c r="B22" s="27" t="s">
+      <c r="A22" s="8"/>
+      <c r="B22" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="31">
+      <c r="C22" s="12">
         <v>100000</v>
       </c>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="27"/>
-      <c r="B23" s="27" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="31">
+      <c r="C23" s="12">
         <v>100000</v>
       </c>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="27"/>
-      <c r="B24" s="27" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="12">
         <v>61746</v>
       </c>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="F24" s="27"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="27"/>
-      <c r="B25" s="27" t="s">
+      <c r="A25" s="8"/>
+      <c r="B25" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="12">
         <v>250000</v>
       </c>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27" t="s">
+      <c r="D25" s="8"/>
+      <c r="E25" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="27"/>
+      <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="27"/>
-      <c r="B26" s="27"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="27"/>
-      <c r="B27" s="27" t="s">
+      <c r="A27" s="8"/>
+      <c r="B27" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="31">
+      <c r="C27" s="12">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4818061D-9312-1C42-9AF7-90E0E6B61A7E}">
+  <dimension ref="B4:I22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="0.5" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="0.5" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:9" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+    </row>
+    <row r="5" spans="2:9" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="I6" s="19"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="C7" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B9" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="34"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B10" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2">
+        <f>'Detailed Cap Table'!C4</f>
+        <v>3600000</v>
+      </c>
+      <c r="D10" s="33"/>
+      <c r="F10" s="4"/>
+      <c r="H10" s="14">
+        <f>C10+F10</f>
+        <v>3600000</v>
+      </c>
+      <c r="I10" s="36">
+        <f>H10/$H$20</f>
+        <v>0.36959987630724139</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B11" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2">
+        <f>'Detailed Cap Table'!C5</f>
+        <v>3600000</v>
+      </c>
+      <c r="D11" s="33"/>
+      <c r="F11" s="4"/>
+      <c r="H11" s="14">
+        <f>C11+F11</f>
+        <v>3600000</v>
+      </c>
+      <c r="I11" s="36">
+        <f>H11/$H$20</f>
+        <v>0.36959987630724139</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B12" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="2">
+        <f>'Detailed Cap Table'!C23-'Detailed Cap Table'!C4-'Detailed Cap Table'!C5+'Detailed Cap Table'!D23-'Detailed Cap Table'!D21+'Detailed Cap Table'!F23</f>
+        <v>2264315</v>
+      </c>
+      <c r="D12" s="33"/>
+      <c r="F12" s="4"/>
+      <c r="H12" s="14">
+        <f>C12+F12</f>
+        <v>2264315</v>
+      </c>
+      <c r="I12" s="36">
+        <f>H12/$H$20</f>
+        <v>0.23246959553350868</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B13" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="2">
+        <f>SUM('Detailed Cap Table'!E4:E20)</f>
+        <v>210843</v>
+      </c>
+      <c r="D13" s="33"/>
+      <c r="F13" s="4"/>
+      <c r="H13" s="14">
+        <f>C13+F13</f>
+        <v>210843</v>
+      </c>
+      <c r="I13" s="36">
+        <f>H13/$H$20</f>
+        <v>2.1646540755624361E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B14" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="33"/>
+      <c r="F14" s="2">
+        <f>'Detailed Cap Table'!D21</f>
+        <v>65105</v>
+      </c>
+      <c r="H14" s="14">
+        <f>C14+F14</f>
+        <v>65105</v>
+      </c>
+      <c r="I14" s="36">
+        <f>H14/$H$20</f>
+        <v>6.6841110963841528E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B15" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="22">
+        <f>SUM(C10:C14)</f>
+        <v>9675158</v>
+      </c>
+      <c r="D15" s="15">
+        <f>SUM(D10:D14)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="22">
+        <f>SUM(F10:F14)</f>
+        <v>65105</v>
+      </c>
+      <c r="H15" s="22">
+        <f>SUM(H10:H14)</f>
+        <v>9740263</v>
+      </c>
+      <c r="I15" s="37">
+        <f>H15/$H$20</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B16" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="33"/>
+      <c r="F16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="29"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B17" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="3">
+        <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
+        <v>8000000</v>
+      </c>
+      <c r="F17" s="4"/>
+      <c r="H17" s="14">
+        <f>C17+F17</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="36">
+        <f>H17/$H$20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B18" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="3">
+        <f>'SAFE Investments'!C27-D17</f>
+        <v>1825000</v>
+      </c>
+      <c r="F18" s="4"/>
+      <c r="H18" s="14">
+        <f>C18+F18</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="36">
+        <f>H18/$H$20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B19" s="7"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="33"/>
+      <c r="F19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="29"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B20" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="27">
+        <f>C15</f>
+        <v>9675158</v>
+      </c>
+      <c r="D20" s="38">
+        <f>SUM(D10:D19)</f>
+        <v>9825000</v>
+      </c>
+      <c r="F20" s="22">
+        <f>F14</f>
+        <v>65105</v>
+      </c>
+      <c r="H20" s="27">
+        <f>SUM(H10:H14)</f>
+        <v>9740263</v>
+      </c>
+      <c r="I20" s="39">
+        <f>SUM(I10:I14)</f>
+        <v>0.99999999999999989</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="7"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="33"/>
+      <c r="F21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="31"/>
+    </row>
+    <row r="22" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" s="30"/>
+      <c r="D22" s="40">
+        <v>50000000</v>
+      </c>
+      <c r="E22" s="6"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Series A fixes applied
</commit_message>
<xml_diff>
--- a/runs/20260414-171016/models/model.xlsx
+++ b/runs/20260414-171016/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86B676E2-B1D6-7C4A-B343-B73AF56EACDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDE8C6A4-570E-6047-B39E-65501EF47CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detailed Cap Table" sheetId="138" r:id="rId1"/>
     <sheet name="SAFE Investments" sheetId="139" r:id="rId2"/>
     <sheet name="Series Seed" sheetId="140" r:id="rId3"/>
+    <sheet name="Series A" sheetId="141" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="88">
   <si>
     <t>Total</t>
   </si>
@@ -202,6 +203,9 @@
     <t xml:space="preserve">Option </t>
   </si>
   <si>
+    <t>Series A</t>
+  </si>
+  <si>
     <t>Total Capitalization</t>
   </si>
   <si>
@@ -211,6 +215,9 @@
     <t>$</t>
   </si>
   <si>
+    <t>Preferred</t>
+  </si>
+  <si>
     <t>Pool +</t>
   </si>
   <si>
@@ -238,9 +245,24 @@
     <t>Total Common</t>
   </si>
   <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>Other Series A Investors</t>
+  </si>
+  <si>
     <t>Totals</t>
   </si>
   <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
     <t>Other Common Shareholders</t>
   </si>
   <si>
@@ -256,20 +278,39 @@
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
   </si>
   <si>
+    <t xml:space="preserve">Price per Share </t>
+  </si>
+  <si>
     <t>SIDEKICK (THINK MORE SECURITY) &amp; 1011 SERIES SEED</t>
   </si>
   <si>
     <t>SAFE Valuation Cap</t>
+  </si>
+  <si>
+    <t>SIDEKICK (THINK MORE SECURITY) &amp; 1011 SERIES A</t>
+  </si>
+  <si>
+    <t>Conversion</t>
+  </si>
+  <si>
+    <t>Expansion</t>
+  </si>
+  <si>
+    <t>Round Ownership %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option Pool Expansion </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0_-;_-[$$-409]* \(#,##0\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.0000_-;_-[$$-409]* \(#,##0.0000\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
   </numFmts>
   <fonts count="25" x14ac:knownFonts="1">
     <font>
@@ -633,7 +674,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -858,6 +899,19 @@
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -909,6 +963,19 @@
         <color rgb="FF000000"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -956,17 +1023,22 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="37" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="37" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -997,13 +1069,19 @@
     <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1012,13 +1090,10 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="37" fontId="20" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1037,13 +1112,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="37" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1061,7 +1145,16 @@
     <xf numFmtId="165" fontId="20" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1473,495 +1566,495 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="8"/>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="A1" s="11"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="9" t="s">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="11"/>
+      <c r="B3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="11"/>
+      <c r="B4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="13">
         <v>3600000</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10">
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="14">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="13">
         <v>3600000</v>
       </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10">
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="14">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="11"/>
+      <c r="B6" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="13">
         <v>222187</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10">
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="14">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="13">
         <v>592500</v>
       </c>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10">
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="14">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8" t="s">
+      <c r="A8" s="11"/>
+      <c r="B8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="13">
         <v>592500</v>
       </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10">
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="14">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="13">
         <v>13500</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="13">
         <v>98900</v>
       </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10">
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="14">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="11"/>
+      <c r="B10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="13">
         <v>9000</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10">
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="14">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13">
         <v>95000</v>
       </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10">
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="14">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10">
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13">
         <v>25000</v>
       </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10">
+      <c r="F12" s="13"/>
+      <c r="G12" s="13">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="14">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10">
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13">
         <v>41562</v>
       </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10">
+      <c r="F13" s="13"/>
+      <c r="G13" s="13">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="14">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8" t="s">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10">
+      <c r="C14" s="13"/>
+      <c r="D14" s="13">
         <v>285000</v>
       </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10">
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="14">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8" t="s">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10">
+      <c r="C15" s="13"/>
+      <c r="D15" s="13">
         <v>50000</v>
       </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10">
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="14">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10">
+      <c r="C16" s="13"/>
+      <c r="D16" s="13">
         <v>285000</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10">
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="14">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8" t="s">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10">
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13">
         <v>96186</v>
       </c>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10">
+      <c r="F17" s="13"/>
+      <c r="G17" s="13">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="11">
+      <c r="H17" s="14">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8" t="s">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10">
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13">
         <v>48095</v>
       </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10">
+      <c r="F18" s="13"/>
+      <c r="G18" s="13">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="11">
+      <c r="H18" s="14">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8" t="s">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10">
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13">
         <v>12395</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="13">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="11">
+      <c r="H19" s="14">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10">
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13">
         <v>8333</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="13">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="11">
+      <c r="H20" s="14">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
     </row>
     <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8" t="s">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10">
+      <c r="C21" s="13"/>
+      <c r="D21" s="13">
         <v>65105</v>
       </c>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10">
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="11">
+      <c r="H21" s="14">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
     </row>
     <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
     </row>
     <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="8"/>
-      <c r="B23" s="9" t="s">
+      <c r="A23" s="11"/>
+      <c r="B23" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="13">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="13">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="13">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F23" s="13">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="13">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="11"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1982,341 +2075,341 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="8"/>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="A1" s="11"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="11"/>
+      <c r="B3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="9" t="s">
+      <c r="D3" s="11"/>
+      <c r="E3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="8"/>
+      <c r="F3" s="11"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="11"/>
+      <c r="B4" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="15">
         <v>25000</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8" t="s">
+      <c r="D4" s="11"/>
+      <c r="E4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="8"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="15">
         <v>25000</v>
       </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="11"/>
+      <c r="B6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="15">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="15">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8" t="s">
+      <c r="A8" s="11"/>
+      <c r="B8" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="15">
         <v>16566</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F8" s="8"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="11"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="15">
         <v>250000</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="11"/>
+      <c r="B10" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="15">
         <v>100000</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="15">
         <v>300000</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8" t="s">
+      <c r="D11" s="11"/>
+      <c r="E11" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="8"/>
+      <c r="F11" s="11"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="15">
         <v>37500</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8" t="s">
+      <c r="D12" s="11"/>
+      <c r="E12" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="8"/>
+      <c r="F12" s="11"/>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="15">
         <v>250000</v>
       </c>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8" t="s">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="15">
         <v>100000</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8" t="s">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="15">
         <v>41164</v>
       </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F15" s="8"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="15">
         <v>2328778</v>
       </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F16" s="8"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="11"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8" t="s">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="15">
         <v>1506000</v>
       </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8" t="s">
+      <c r="D17" s="11"/>
+      <c r="E17" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="8"/>
+      <c r="F17" s="11"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8" t="s">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="15">
         <v>50000</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8" t="s">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="15">
         <v>212500</v>
       </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8" t="s">
+      <c r="D19" s="11"/>
+      <c r="E19" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="8"/>
+      <c r="F19" s="11"/>
     </row>
     <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="15">
         <v>25000</v>
       </c>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8" t="s">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="15">
         <v>61746</v>
       </c>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F21" s="8"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F21" s="11"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8" t="s">
+      <c r="A22" s="11"/>
+      <c r="B22" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="15">
         <v>100000</v>
       </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8" t="s">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="15">
         <v>100000</v>
       </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="15">
         <v>61746</v>
       </c>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F24" s="8"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F24" s="11"/>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8" t="s">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="12">
+      <c r="C25" s="15">
         <v>250000</v>
       </c>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8" t="s">
+      <c r="D25" s="11"/>
+      <c r="E25" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="8"/>
+      <c r="F25" s="11"/>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
+      <c r="A26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8" t="s">
+      <c r="A27" s="11"/>
+      <c r="B27" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="15">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2341,301 +2434,857 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:9" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
+      <c r="B4" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
     </row>
     <row r="5" spans="2:9" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="I6" s="19"/>
+      <c r="H6" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="I6" s="23"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="C7" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="21" t="s">
+      <c r="C7" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="D7" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" s="19" t="s">
+      <c r="F7" s="24" t="s">
         <v>60</v>
       </c>
+      <c r="H7" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="8" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" s="20" t="s">
+      <c r="C8" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="H8" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="I8" s="17" t="s">
+      <c r="D8" s="24" t="s">
         <v>64</v>
       </c>
+      <c r="F8" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" s="21" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="34"/>
+      <c r="B9" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="39"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="4">
         <f>'Detailed Cap Table'!C4</f>
         <v>3600000</v>
       </c>
-      <c r="D10" s="33"/>
-      <c r="F10" s="4"/>
-      <c r="H10" s="14">
+      <c r="D10" s="38"/>
+      <c r="F10" s="7"/>
+      <c r="H10" s="17">
         <f>C10+F10</f>
         <v>3600000</v>
       </c>
-      <c r="I10" s="36">
+      <c r="I10" s="43">
         <f>H10/$H$20</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="4">
         <f>'Detailed Cap Table'!C5</f>
         <v>3600000</v>
       </c>
-      <c r="D11" s="33"/>
-      <c r="F11" s="4"/>
-      <c r="H11" s="14">
+      <c r="D11" s="38"/>
+      <c r="F11" s="7"/>
+      <c r="H11" s="17">
         <f>C11+F11</f>
         <v>3600000</v>
       </c>
-      <c r="I11" s="36">
+      <c r="I11" s="43">
         <f>H11/$H$20</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B12" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="2">
+      <c r="B12" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="4">
         <f>'Detailed Cap Table'!C23-'Detailed Cap Table'!C4-'Detailed Cap Table'!C5+'Detailed Cap Table'!D23-'Detailed Cap Table'!D21+'Detailed Cap Table'!F23</f>
         <v>2264315</v>
       </c>
-      <c r="D12" s="33"/>
-      <c r="F12" s="4"/>
-      <c r="H12" s="14">
+      <c r="D12" s="38"/>
+      <c r="F12" s="7"/>
+      <c r="H12" s="17">
         <f>C12+F12</f>
         <v>2264315</v>
       </c>
-      <c r="I12" s="36">
+      <c r="I12" s="43">
         <f>H12/$H$20</f>
         <v>0.23246959553350868</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="2">
+      <c r="B13" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="4">
         <f>SUM('Detailed Cap Table'!E4:E20)</f>
         <v>210843</v>
       </c>
-      <c r="D13" s="33"/>
-      <c r="F13" s="4"/>
-      <c r="H13" s="14">
+      <c r="D13" s="38"/>
+      <c r="F13" s="7"/>
+      <c r="H13" s="17">
         <f>C13+F13</f>
         <v>210843</v>
       </c>
-      <c r="I13" s="36">
+      <c r="I13" s="43">
         <f>H13/$H$20</f>
         <v>2.1646540755624361E-2</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="33"/>
-      <c r="F14" s="2">
+      <c r="B14" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="4">
         <f>'Detailed Cap Table'!D21</f>
         <v>65105</v>
       </c>
-      <c r="H14" s="14">
+      <c r="D14" s="38"/>
+      <c r="H14" s="17">
         <f>C14+F14</f>
         <v>65105</v>
       </c>
-      <c r="I14" s="36">
+      <c r="I14" s="43">
         <f>H14/$H$20</f>
         <v>6.6841110963841528E-3</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B15" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" s="22">
+      <c r="B15" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="26">
         <f>SUM(C10:C14)</f>
-        <v>9675158</v>
-      </c>
-      <c r="D15" s="15">
+        <v>9740263</v>
+      </c>
+      <c r="D15" s="18">
         <f>SUM(D10:D14)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="26">
         <f>SUM(F10:F14)</f>
-        <v>65105</v>
-      </c>
-      <c r="H15" s="22">
+        <v>0</v>
+      </c>
+      <c r="H15" s="26">
         <f>SUM(H10:H14)</f>
         <v>9740263</v>
       </c>
-      <c r="I15" s="37">
+      <c r="I15" s="44">
         <f>H15/$H$20</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="33"/>
-      <c r="F16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="29"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="38"/>
+      <c r="F16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="33"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="3">
+      <c r="C17" s="7"/>
+      <c r="D17" s="5">
         <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
         <v>8000000</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="H17" s="14">
+      <c r="F17" s="7"/>
+      <c r="H17" s="17">
         <f>C17+F17</f>
         <v>0</v>
       </c>
-      <c r="I17" s="36">
+      <c r="I17" s="43">
         <f>H17/$H$20</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B18" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="3">
+      <c r="B18" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="5">
         <f>'SAFE Investments'!C27-D17</f>
         <v>1825000</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="H18" s="14">
+      <c r="F18" s="7"/>
+      <c r="H18" s="17">
         <f>C18+F18</f>
         <v>0</v>
       </c>
-      <c r="I18" s="36">
+      <c r="I18" s="43">
         <f>H18/$H$20</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="7"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="33"/>
-      <c r="F19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="29"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="38"/>
+      <c r="F19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="33"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="27">
+      <c r="B20" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="31">
         <f>C15</f>
-        <v>9675158</v>
-      </c>
-      <c r="D20" s="38">
+        <v>9740263</v>
+      </c>
+      <c r="D20" s="45">
         <f>SUM(D10:D19)</f>
         <v>9825000</v>
       </c>
-      <c r="F20" s="22">
-        <f>F14</f>
-        <v>65105</v>
-      </c>
-      <c r="H20" s="27">
+      <c r="F20" s="26">
+        <f>F15</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="31">
         <f>SUM(H10:H14)</f>
         <v>9740263</v>
       </c>
-      <c r="I20" s="39">
+      <c r="I20" s="46">
         <f>SUM(I10:I14)</f>
         <v>0.99999999999999989</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="7"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="33"/>
-      <c r="F21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="31"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="38"/>
+      <c r="F21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="35"/>
     </row>
     <row r="22" spans="2:9" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" s="34"/>
+      <c r="D22" s="47">
+        <v>50000000</v>
+      </c>
+      <c r="E22" s="9"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="37"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18BBD0FB-B3E3-4C45-B342-508DD1173A95}">
+  <dimension ref="B2:O28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" customWidth="1"/>
+    <col min="13" max="13" width="0.5" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" customWidth="1"/>
+    <col min="16" max="16" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+    </row>
+    <row r="3" spans="2:15" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="48"/>
+      <c r="G4" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="23"/>
+      <c r="L4" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="O4" s="23"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="C5" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="L5" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="N5" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="O5" s="23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L6" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="N6" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="O6" s="21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B7" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="39"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B8" s="28" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4">
+        <f>'Series Seed'!C10</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="38"/>
+      <c r="E8" s="17"/>
+      <c r="G8" s="7"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="17"/>
+      <c r="L8" s="17"/>
+      <c r="N8" s="17">
+        <f>C8+E8+G8+J8+L8</f>
+        <v>3600000</v>
+      </c>
+      <c r="O8" s="43">
+        <f ca="1">N8/$N$19</f>
+        <v>0.18701982455766836</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B9" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="4">
+        <f>'Series Seed'!C11</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="38"/>
+      <c r="E9" s="17"/>
+      <c r="G9" s="7"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="17"/>
+      <c r="L9" s="17"/>
+      <c r="N9" s="17">
+        <f>C9+E9+G9+J9+L9</f>
+        <v>3600000</v>
+      </c>
+      <c r="O9" s="43">
+        <f ca="1">N9/$N$19</f>
+        <v>0.18701982455766836</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B10" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="4">
+        <f>'Series Seed'!C12</f>
+        <v>2264315</v>
+      </c>
+      <c r="D10" s="38"/>
+      <c r="E10" s="17"/>
+      <c r="G10" s="7"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="N10" s="17">
+        <f>C10+E10+G10+J10+L10</f>
+        <v>2264315</v>
+      </c>
+      <c r="O10" s="43">
+        <f ca="1">N10/$N$19</f>
+        <v>0.11763105390091579</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="4">
+        <f>'Series Seed'!C13</f>
+        <v>210843</v>
+      </c>
+      <c r="D11" s="38"/>
+      <c r="E11" s="17"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="N11" s="17">
+        <f>C11+E11+G11+J11+L11</f>
+        <v>210843</v>
+      </c>
+      <c r="O11" s="43">
+        <f ca="1">N11/$N$19</f>
+        <v>1.0953283574781241E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B12" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="4">
+        <f>'Series Seed'!C14</f>
+        <v>65105</v>
+      </c>
+      <c r="D12" s="38"/>
+      <c r="E12" s="17"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="17"/>
+      <c r="L12" s="17">
+        <f ca="1">IFERROR(ROUNDDOWN(0.1*N19-C12,0),0)</f>
+        <v>1859824</v>
+      </c>
+      <c r="N12" s="17">
+        <f ca="1">C12+E12+G12+J12+L12</f>
+        <v>1924929</v>
+      </c>
+      <c r="O12" s="43">
+        <f ca="1">N12/$N$19</f>
+        <v>9.9999967740546661E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B13" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="36">
+        <f>SUM(C8:C12)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D13" s="38">
+        <f>SUM(D8:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="17">
+        <f>SUM(E8:E12)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="36">
+        <f>SUM(G8:G12)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="38">
+        <f>SUM(I8:I12)</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="17">
+        <f>SUM(J8:J12)</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="26">
+        <f ca="1">SUM(L8:L12)</f>
+        <v>1859824</v>
+      </c>
+      <c r="N13" s="26">
+        <f ca="1">SUM(N8:N12)</f>
+        <v>11600087</v>
+      </c>
+      <c r="O13" s="44">
+        <f ca="1">N13/$N$19</f>
+        <v>0.60262395433158045</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B14" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="17"/>
+      <c r="G14" s="7"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="43"/>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B15" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="5">
+        <f>'Series Seed'!D17</f>
+        <v>8000000</v>
+      </c>
+      <c r="E15" s="17">
+        <f ca="1">D15/$E$21</f>
+        <v>2309935.6105448562</v>
+      </c>
+      <c r="G15" s="7"/>
+      <c r="I15" s="3">
+        <v>5000000</v>
+      </c>
+      <c r="J15" s="17">
+        <f ca="1">I15/$J$21</f>
+        <v>1203079.8845043313</v>
+      </c>
+      <c r="L15" s="17"/>
+      <c r="N15" s="17">
+        <f ca="1">C15+E15+G15+J15+L15</f>
+        <v>3513015.4950491874</v>
+      </c>
+      <c r="O15" s="43">
+        <f ca="1">N15/$N$19</f>
+        <v>0.18250098376457485</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B16" s="28">
+        <v>1011</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="17"/>
+      <c r="G16" s="7"/>
+      <c r="I16" s="3">
+        <v>12000000</v>
+      </c>
+      <c r="J16" s="17">
+        <f ca="1">I16/$J$21</f>
+        <v>2887391.7228103946</v>
+      </c>
+      <c r="L16" s="17"/>
+      <c r="N16" s="17">
+        <f ca="1">C16+E16+G16+J16+L16</f>
+        <v>2887391.7228103946</v>
+      </c>
+      <c r="O16" s="43">
+        <f ca="1">N16/$N$19</f>
+        <v>0.14999985928590662</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B17" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="17"/>
+      <c r="G17" s="7"/>
+      <c r="I17" s="3">
+        <v>3000000</v>
+      </c>
+      <c r="J17" s="17">
+        <f ca="1">I17/$J$21</f>
+        <v>721847.93070259865</v>
+      </c>
+      <c r="L17" s="17"/>
+      <c r="N17" s="17">
+        <f ca="1">C17+E17+G17+J17+L17</f>
+        <v>721847.93070259865</v>
+      </c>
+      <c r="O17" s="43">
+        <f ca="1">N17/$N$19</f>
+        <v>3.7499964821476654E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B18" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="5">
+        <f>'Series Seed'!D18</f>
+        <v>1825000</v>
+      </c>
+      <c r="E18" s="17">
+        <f ca="1">D18/$E$21</f>
+        <v>526954.06115554529</v>
+      </c>
+      <c r="G18" s="7"/>
+      <c r="I18" s="38"/>
+      <c r="J18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="N18" s="17">
+        <f ca="1">C18+E18+G18+J18+L18</f>
+        <v>526954.06115554529</v>
+      </c>
+      <c r="O18" s="43">
+        <f ca="1">N18/$N$19</f>
+        <v>2.7375237796461366E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B19" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="49">
+        <f>C13</f>
+        <v>9740263</v>
+      </c>
+      <c r="D19" s="50">
+        <f>SUM(D8:D18)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E19" s="31">
+        <f ca="1">SUM(E8:E18)</f>
+        <v>2836889.6717004012</v>
+      </c>
+      <c r="G19" s="36">
+        <f>SUM(G8:G18)</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="50">
+        <f>SUM(I8:I18)</f>
+        <v>20000000</v>
+      </c>
+      <c r="J19" s="31">
+        <f ca="1">SUM(J8:J18)</f>
+        <v>4812319.5380173242</v>
+      </c>
+      <c r="L19" s="26">
+        <f ca="1">L12</f>
+        <v>1859824</v>
+      </c>
+      <c r="N19" s="31">
+        <f ca="1">SUM(N15:N18)+N13</f>
+        <v>19249296.209717728</v>
+      </c>
+      <c r="O19" s="46">
+        <f ca="1">SUM(O15:O18)+O13</f>
+        <v>0.99999999999999989</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="10"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="35"/>
+    </row>
+    <row r="21" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="40">
+        <f ca="1">IFERROR(ROUND((50000000-D19)/(C19+L12),4),0)</f>
+        <v>3.4632999999999998</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="40">
+        <f ca="1">IFERROR(ROUND(J22/(C19+E19+G19+L19),4),0)</f>
+        <v>4.1559999999999997</v>
+      </c>
+      <c r="L21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="35"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B22" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="3">
+        <v>60000000</v>
+      </c>
+      <c r="L22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="35"/>
+    </row>
+    <row r="23" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="34"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="34"/>
+      <c r="J23" s="41">
+        <f>J22+I19</f>
+        <v>80000000</v>
+      </c>
+      <c r="K23" s="9"/>
+      <c r="L23" s="34"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="34"/>
+      <c r="O23" s="37"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B25" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="40">
-        <v>50000000</v>
-      </c>
-      <c r="E22" s="6"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="32"/>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B27" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="1">
+        <f>I19/J23</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="28" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B28" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" s="1">
+        <f ca="1">IFERROR(0.1-(G12/N19),0)</f>
+        <v>0.1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Sheet 3: Series Seed with grouped shareholders
</commit_message>
<xml_diff>
--- a/runs/20260414-171016/models/model.xlsx
+++ b/runs/20260414-171016/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D021136-4E76-0F42-879F-CBC79C837084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F966789-D82A-AE47-91D4-5E8BC370B65E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="143" r:id="rId1"/>
     <sheet name="Detailed Cap Table" sheetId="144" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="145" r:id="rId3"/>
+    <sheet name="Series Seed" sheetId="146" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="79">
   <si>
     <t>Total</t>
   </si>
@@ -193,17 +194,97 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t>SIDEKICK (THINK MORE SECURITY, INC.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option </t>
+  </si>
+  <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Other Common Shareholders</t>
+  </si>
+  <si>
+    <t>ESOP Issued &amp; Outstanding</t>
+  </si>
+  <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
+    <t>Other SAFE Investors</t>
+  </si>
+  <si>
+    <t>Invested</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% </t>
+  </si>
+  <si>
+    <t>SAFE Valuation Cap</t>
+  </si>
+  <si>
+    <t>Pre-Funding</t>
+  </si>
+  <si>
+    <t>Val Cap</t>
+  </si>
+  <si>
+    <t>($)</t>
+  </si>
+  <si>
+    <t>SAFE Rounds</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation Cap</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0_-;_-[$$-409]* \(#,##0\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -339,6 +420,39 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -351,6 +465,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -533,7 +654,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -648,6 +769,141 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -693,8 +949,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -704,24 +961,84 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1141,610 +1458,610 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="5" t="s">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="4"/>
+      <c r="B3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="4"/>
+      <c r="B4" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="23">
         <v>3600000</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6">
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="24">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="4"/>
+      <c r="B5" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="23">
         <v>3600000</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6">
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="24">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="23">
         <v>222187</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6">
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="24">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="23">
         <v>592500</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6">
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="24">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="23">
         <v>592500</v>
       </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6">
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="24">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="23">
         <v>13500</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="23">
         <v>98900</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6">
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="24">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="4"/>
+      <c r="B10" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="23">
         <v>9000</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6">
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="24">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6">
+      <c r="C11" s="23"/>
+      <c r="D11" s="23">
         <v>95000</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6">
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="24">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="4"/>
+      <c r="B12" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6">
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23">
         <v>25000</v>
       </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6">
+      <c r="F12" s="23"/>
+      <c r="G12" s="23">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="24">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="4"/>
+      <c r="B13" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6">
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23">
         <v>41562</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6">
+      <c r="F13" s="23"/>
+      <c r="G13" s="23">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="24">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="4"/>
+      <c r="B14" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6">
+      <c r="C14" s="23"/>
+      <c r="D14" s="23">
         <v>285000</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6">
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="24">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="4"/>
+      <c r="B15" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6">
+      <c r="C15" s="23"/>
+      <c r="D15" s="23">
         <v>50000</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6">
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="24">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="4"/>
+      <c r="B16" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6">
+      <c r="C16" s="23"/>
+      <c r="D16" s="23">
         <v>285000</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6">
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="24">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="4"/>
+      <c r="B17" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6">
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23">
         <v>96186</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6">
+      <c r="F17" s="23"/>
+      <c r="G17" s="23">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="24">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4" t="s">
+      <c r="A18" s="4"/>
+      <c r="B18" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6">
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23">
         <v>48095</v>
       </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6">
+      <c r="F18" s="23"/>
+      <c r="G18" s="23">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="24">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4" t="s">
+      <c r="A19" s="4"/>
+      <c r="B19" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6">
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23">
         <v>12395</v>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="23">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="24">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4" t="s">
+      <c r="A20" s="4"/>
+      <c r="B20" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6">
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23">
         <v>8333</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="23">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="24">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
     </row>
     <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4" t="s">
+      <c r="A21" s="4"/>
+      <c r="B21" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6">
+      <c r="C21" s="23"/>
+      <c r="D21" s="23">
         <v>65105</v>
       </c>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6">
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="24">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
-      <c r="O21" s="3"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
-      <c r="O22" s="3"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="4"/>
+      <c r="B23" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="23">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="23">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="23">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="23">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="23">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1765,476 +2082,965 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="4"/>
+      <c r="B3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="5" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="4"/>
+      <c r="B4" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="26">
         <v>25000</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="4"/>
+      <c r="B5" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="26">
         <v>25000</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="26">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="26">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="26">
         <v>16566</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="26">
         <v>250000</v>
       </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="4"/>
+      <c r="B10" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="26">
         <v>100000</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="26">
         <v>300000</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="4" t="s">
+      <c r="D11" s="4"/>
+      <c r="E11" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="4"/>
+      <c r="B12" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="26">
         <v>37500</v>
       </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="4" t="s">
+      <c r="D12" s="4"/>
+      <c r="E12" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="4"/>
+      <c r="B13" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="26">
         <v>250000</v>
       </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="4"/>
+      <c r="B14" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="26">
         <v>100000</v>
       </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="4"/>
+      <c r="B15" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="26">
         <v>41164</v>
       </c>
-      <c r="D15" s="3"/>
-      <c r="E15" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="4"/>
+      <c r="B16" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="26">
         <v>2328778</v>
       </c>
-      <c r="D16" s="3"/>
-      <c r="E16" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="4"/>
+      <c r="B17" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="26">
         <v>1506000</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="4" t="s">
+      <c r="D17" s="4"/>
+      <c r="E17" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4" t="s">
+      <c r="A18" s="4"/>
+      <c r="B18" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="26">
         <v>50000</v>
       </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4" t="s">
+      <c r="A19" s="4"/>
+      <c r="B19" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="26">
         <v>212500</v>
       </c>
-      <c r="D19" s="3"/>
-      <c r="E19" s="4" t="s">
+      <c r="D19" s="4"/>
+      <c r="E19" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4" t="s">
+      <c r="A20" s="4"/>
+      <c r="B20" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="26">
         <v>25000</v>
       </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4" t="s">
+      <c r="A21" s="4"/>
+      <c r="B21" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="26">
         <v>61746</v>
       </c>
-      <c r="D21" s="3"/>
-      <c r="E21" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="4"/>
+      <c r="B22" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="26">
         <v>100000</v>
       </c>
-      <c r="D22" s="3"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4" t="s">
+      <c r="A23" s="4"/>
+      <c r="B23" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="26">
         <v>100000</v>
       </c>
-      <c r="D23" s="3"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="3"/>
-      <c r="B24" s="4" t="s">
+      <c r="A24" s="4"/>
+      <c r="B24" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="26">
         <v>61746</v>
       </c>
-      <c r="D24" s="3"/>
-      <c r="E24" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="3"/>
-      <c r="B25" s="4" t="s">
+      <c r="A25" s="4"/>
+      <c r="B25" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="26">
         <v>250000</v>
       </c>
-      <c r="D25" s="3"/>
-      <c r="E25" s="4" t="s">
+      <c r="D25" s="4"/>
+      <c r="E25" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="3"/>
-      <c r="B27" s="4" t="s">
+      <c r="A27" s="4"/>
+      <c r="B27" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="25">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9B24787-5B03-6349-A875-B2FF2EAE12B3}">
+  <dimension ref="B1:N25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="15.5" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="0.5" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" customWidth="1"/>
+    <col min="13" max="13" width="9.33203125" customWidth="1"/>
+    <col min="14" max="14" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="8"/>
+    </row>
+    <row r="2" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="8"/>
+    </row>
+    <row r="4" spans="2:14" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="8"/>
+    </row>
+    <row r="5" spans="2:14" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="8"/>
+    </row>
+    <row r="6" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="17"/>
+      <c r="E6" s="37"/>
+      <c r="G6" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="37"/>
+      <c r="J6" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K6" s="13"/>
+      <c r="L6" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" s="37"/>
+      <c r="N6" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C7" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="40" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="G7" s="40" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="K7" s="33"/>
+      <c r="L7" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="M7" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="J8" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="33"/>
+      <c r="L8" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="M8" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B9" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="35"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B10" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="6">
+        <f>'Detailed Cap Table'!C4</f>
+        <v>3600000</v>
+      </c>
+      <c r="E10" s="1"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="L10" s="27">
+        <f>C10+E10+H10+J10</f>
+        <v>3600000</v>
+      </c>
+      <c r="M10" s="41">
+        <f>L10/$L$21</f>
+        <v>0.36959987630724139</v>
+      </c>
+      <c r="N10" s="38">
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B11" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6">
+        <f>'Detailed Cap Table'!C5</f>
+        <v>3600000</v>
+      </c>
+      <c r="E11" s="1"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="L11" s="27">
+        <f>C11+E11+H11+J11</f>
+        <v>3600000</v>
+      </c>
+      <c r="M11" s="41">
+        <f>L11/$L$21</f>
+        <v>0.36959987630724139</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="6">
+        <f>SUM('Detailed Cap Table'!C6:'Detailed Cap Table'!C10)</f>
+        <v>1429687</v>
+      </c>
+      <c r="E12" s="1"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="L12" s="27">
+        <f>C12+E12+H12+J12</f>
+        <v>1429687</v>
+      </c>
+      <c r="M12" s="41">
+        <f>L12/$L$21</f>
+        <v>0.14678114954390861</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B13" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="6">
+        <f>'Detailed Cap Table'!D9+'Detailed Cap Table'!D11+'Detailed Cap Table'!D14+'Detailed Cap Table'!D15+'Detailed Cap Table'!D16+'Detailed Cap Table'!E12+'Detailed Cap Table'!E13+'Detailed Cap Table'!E17+'Detailed Cap Table'!E18+'Detailed Cap Table'!F19+'Detailed Cap Table'!F20</f>
+        <v>1045471</v>
+      </c>
+      <c r="E13" s="1"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="L13" s="27">
+        <f>C13+E13+H13+J13</f>
+        <v>1045471</v>
+      </c>
+      <c r="M13" s="41">
+        <f>L13/$L$21</f>
+        <v>0.10733498674522443</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B14" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="6">
+        <f>'Detailed Cap Table'!D21</f>
+        <v>65105</v>
+      </c>
+      <c r="E14" s="1"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="L14" s="27">
+        <f>C14+E14+H14+J14</f>
+        <v>65105</v>
+      </c>
+      <c r="M14" s="41">
+        <f>L14/$L$21</f>
+        <v>6.6841110963841528E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B15" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="43">
+        <f>SUM(C10:C14)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D15">
+        <f>SUM(D10:D14)</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <f>SUM(E10:E14)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="10">
+        <f>SUM(G10:G14)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <f>SUM(H10:H14)</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="43">
+        <f>SUM(J10:J14)</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="43">
+        <f>SUM(L10:L14)</f>
+        <v>9740263</v>
+      </c>
+      <c r="M15" s="44">
+        <f>L15/$L$21</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B16" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="42"/>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B17" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="G17" s="36">
+        <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
+        <v>8000000</v>
+      </c>
+      <c r="H17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="L17" s="27">
+        <f>C17+E17+H17+J17</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="41">
+        <f>L17/$L$21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B18" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="G18" s="36">
+        <f>'SAFE Investments'!C27-G17</f>
+        <v>1825000</v>
+      </c>
+      <c r="H18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="L18" s="27">
+        <f>C18+E18+H18+J18</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="41">
+        <f>L18/$L$21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B19" s="13"/>
+      <c r="C19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="42"/>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B20" s="13"/>
+      <c r="C20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="42"/>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B21" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="45">
+        <f>C15+SUM(C17:C18)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D21" s="31">
+        <f>SUM(D10:D20)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="45">
+        <f>SUM(E10:E20)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="46">
+        <f>SUM(G10:G20)</f>
+        <v>9825000</v>
+      </c>
+      <c r="H21" s="45">
+        <f>SUM(H10:H20)</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="43">
+        <f>J14</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="45">
+        <f>SUM(L17:L20)+L15</f>
+        <v>9740263</v>
+      </c>
+      <c r="M21" s="47">
+        <f>SUM(M17:M18)+M15</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="13"/>
+      <c r="M22" s="15"/>
+    </row>
+    <row r="23" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="M23" s="15"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B24" s="13"/>
+      <c r="M24" s="15"/>
+    </row>
+    <row r="25" spans="2:13" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="48">
+        <v>50000000</v>
+      </c>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Sheet 4: Series A with SAFE conversion and option pool expansion
</commit_message>
<xml_diff>
--- a/runs/20260414-171016/models/model.xlsx
+++ b/runs/20260414-171016/models/model.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F966789-D82A-AE47-91D4-5E8BC370B65E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2419F7D4-6A8B-3C49-8C12-A100E19F55BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="143" r:id="rId1"/>
     <sheet name="Detailed Cap Table" sheetId="144" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="145" r:id="rId3"/>
     <sheet name="Series Seed" sheetId="146" r:id="rId4"/>
+    <sheet name="Series A" sheetId="147" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="96">
   <si>
     <t>Total</t>
   </si>
@@ -203,6 +204,9 @@
     <t xml:space="preserve">Option </t>
   </si>
   <si>
+    <t>Series A</t>
+  </si>
+  <si>
     <t>Total Capitalization</t>
   </si>
   <si>
@@ -224,6 +228,9 @@
     <t>Shares</t>
   </si>
   <si>
+    <t>Pre A</t>
+  </si>
+  <si>
     <t>FD</t>
   </si>
   <si>
@@ -233,9 +240,36 @@
     <t>Total Common</t>
   </si>
   <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>1011 Ventures</t>
+  </si>
+  <si>
+    <t>Other Series A Investors</t>
+  </si>
+  <si>
     <t>Totals</t>
   </si>
   <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
+    <t>Total Raised</t>
+  </si>
+  <si>
+    <t>% Ownership</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation Step-up</t>
+  </si>
+  <si>
     <t>Other Common Shareholders</t>
   </si>
   <si>
@@ -251,15 +285,30 @@
     <t>Invested</t>
   </si>
   <si>
+    <t>Post A</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
   </si>
   <si>
     <t xml:space="preserve">% </t>
   </si>
   <si>
+    <t>1011 Contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price per Share </t>
+  </si>
+  <si>
+    <t>SAFE Conversion</t>
+  </si>
+  <si>
     <t>SAFE Valuation Cap</t>
   </si>
   <si>
+    <t>Option Pool Expansion %</t>
+  </si>
+  <si>
     <t>Pre-Funding</t>
   </si>
   <si>
@@ -273,18 +322,23 @@
   </si>
   <si>
     <t>Post-Money Valuation Cap</t>
+  </si>
+  <si>
+    <t>SERIES A ROUND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0_-;_-[$$-409]* \(#,##0\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.0000_-;_-[$$-409]* \(#,##0.0000\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -427,9 +481,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Garamond"/>
       <family val="1"/>
     </font>
@@ -473,7 +539,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -653,8 +719,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -889,6 +961,34 @@
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -949,8 +1049,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -961,67 +1062,74 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="21" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1031,7 +1139,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1039,6 +1147,12 @@
     <xf numFmtId="168" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="178" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="178" fontId="21" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="21" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1458,610 +1572,610 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="22" t="s">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
-      <c r="B3" s="22" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
-      <c r="B4" s="21" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C4" s="28">
         <v>3600000</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23">
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="24">
+      <c r="H4" s="29">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="28">
         <v>3600000</v>
       </c>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23">
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="29">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
-      <c r="B6" s="21" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="28">
         <v>222187</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23">
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="29">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="4"/>
-      <c r="B7" s="21" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="28">
         <v>592500</v>
       </c>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23">
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="29">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="B8" s="21" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="28">
         <v>592500</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23">
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="29">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
-      <c r="B9" s="21" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="28">
         <v>13500</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="28">
         <v>98900</v>
       </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23">
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="24">
+      <c r="H9" s="29">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="21" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="28">
         <v>9000</v>
       </c>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23">
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="29">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23">
+      <c r="C11" s="28"/>
+      <c r="D11" s="28">
         <v>95000</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23">
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="29">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="21" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23">
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28">
         <v>25000</v>
       </c>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23">
+      <c r="F12" s="28"/>
+      <c r="G12" s="28">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="29">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="4"/>
-      <c r="B13" s="21" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23">
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28">
         <v>41562</v>
       </c>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23">
+      <c r="F13" s="28"/>
+      <c r="G13" s="28">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="29">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="21" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23">
+      <c r="C14" s="28"/>
+      <c r="D14" s="28">
         <v>285000</v>
       </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23">
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="29">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
-      <c r="B15" s="21" t="s">
+      <c r="A15" s="5"/>
+      <c r="B15" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23">
+      <c r="C15" s="28"/>
+      <c r="D15" s="28">
         <v>50000</v>
       </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23">
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="29">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="21" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23">
+      <c r="C16" s="28"/>
+      <c r="D16" s="28">
         <v>285000</v>
       </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23">
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="24">
+      <c r="H16" s="29">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="21" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23">
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28">
         <v>96186</v>
       </c>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23">
+      <c r="F17" s="28"/>
+      <c r="G17" s="28">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="29">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="21" t="s">
+      <c r="A18" s="5"/>
+      <c r="B18" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23">
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28">
         <v>48095</v>
       </c>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23">
+      <c r="F18" s="28"/>
+      <c r="G18" s="28">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="24">
+      <c r="H18" s="29">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
-      <c r="B19" s="21" t="s">
+      <c r="A19" s="5"/>
+      <c r="B19" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23">
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28">
         <v>12395</v>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="28">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="29">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="21" t="s">
+      <c r="A20" s="5"/>
+      <c r="B20" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23">
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28">
         <v>8333</v>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="28">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="24">
+      <c r="H20" s="29">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
     </row>
     <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
-      <c r="B21" s="21" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23">
+      <c r="C21" s="28"/>
+      <c r="D21" s="28">
         <v>65105</v>
       </c>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23">
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="24">
+      <c r="H21" s="29">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-      <c r="B23" s="22" t="s">
+      <c r="A23" s="5"/>
+      <c r="B23" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="23">
+      <c r="C23" s="28">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="28">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="28">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="23">
+      <c r="F23" s="28">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="23">
+      <c r="G23" s="28">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2082,476 +2196,476 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
-      <c r="B3" s="22" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="22" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
-      <c r="B4" s="21" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="31">
         <v>25000</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="21" t="s">
+      <c r="D4" s="5"/>
+      <c r="E4" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="31">
         <v>25000</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
-      <c r="B6" s="21" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="31">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4"/>
-      <c r="B7" s="21" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="31">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="B8" s="21" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="31">
         <v>16566</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
-      <c r="B9" s="21" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="31">
         <v>250000</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="21" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="31">
         <v>100000</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="31">
         <v>300000</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="21" t="s">
+      <c r="D11" s="5"/>
+      <c r="E11" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="21" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="31">
         <v>37500</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="21" t="s">
+      <c r="D12" s="5"/>
+      <c r="E12" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="4"/>
-      <c r="B13" s="21" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="31">
         <v>250000</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="21" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="31">
         <v>100000</v>
       </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
-      <c r="B15" s="21" t="s">
+      <c r="A15" s="5"/>
+      <c r="B15" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="31">
         <v>41164</v>
       </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="21" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="31">
         <v>2328778</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="21" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="31">
         <v>1506000</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="21" t="s">
+      <c r="D17" s="5"/>
+      <c r="E17" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="21" t="s">
+      <c r="A18" s="5"/>
+      <c r="B18" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="31">
         <v>50000</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
-      <c r="B19" s="21" t="s">
+      <c r="A19" s="5"/>
+      <c r="B19" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="26">
+      <c r="C19" s="31">
         <v>212500</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="21" t="s">
+      <c r="D19" s="5"/>
+      <c r="E19" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="21" t="s">
+      <c r="A20" s="5"/>
+      <c r="B20" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="26">
+      <c r="C20" s="31">
         <v>25000</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
-      <c r="B21" s="21" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="26">
+      <c r="C21" s="31">
         <v>61746</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="21" t="s">
+      <c r="A22" s="5"/>
+      <c r="B22" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="31">
         <v>100000</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-      <c r="B23" s="21" t="s">
+      <c r="A23" s="5"/>
+      <c r="B23" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="26">
+      <c r="C23" s="31">
         <v>100000</v>
       </c>
-      <c r="D23" s="4"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
-      <c r="B24" s="21" t="s">
+      <c r="A24" s="5"/>
+      <c r="B24" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="26">
+      <c r="C24" s="31">
         <v>61746</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="4"/>
-      <c r="B25" s="21" t="s">
+      <c r="A25" s="5"/>
+      <c r="B25" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="31">
         <v>250000</v>
       </c>
-      <c r="D25" s="4"/>
-      <c r="E25" s="21" t="s">
+      <c r="D25" s="5"/>
+      <c r="E25" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="4"/>
-      <c r="B27" s="21" t="s">
+      <c r="A27" s="5"/>
+      <c r="B27" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="25">
+      <c r="C27" s="30">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2576,297 +2690,297 @@
     <col min="11" max="11" width="0.5" customWidth="1"/>
     <col min="12" max="12" width="14.33203125" customWidth="1"/>
     <col min="13" max="13" width="9.33203125" customWidth="1"/>
-    <col min="14" max="14" width="8" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="8"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="11"/>
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="8"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="11"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="8"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="11"/>
     </row>
     <row r="4" spans="2:14" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="8"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="11"/>
     </row>
     <row r="5" spans="2:14" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="N5" s="8"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="11"/>
     </row>
     <row r="6" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="37"/>
-      <c r="G6" s="17" t="s">
+      <c r="D6" s="21"/>
+      <c r="E6" s="43"/>
+      <c r="G6" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="37"/>
-      <c r="J6" s="17" t="s">
+      <c r="H6" s="43"/>
+      <c r="J6" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="13"/>
-      <c r="L6" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="M6" s="37"/>
-      <c r="N6" s="5" t="s">
+      <c r="K6" s="17"/>
+      <c r="L6" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M6" s="43"/>
+      <c r="N6" s="7" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C7" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="40" t="s">
+      <c r="C7" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="D7" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="40" t="s">
-        <v>57</v>
-      </c>
-      <c r="H7" s="20" t="s">
+      <c r="E7" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="J7" s="19" t="s">
+      <c r="H7" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="K7" s="33"/>
-      <c r="L7" s="17" t="s">
+      <c r="J7" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="M7" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>75</v>
+      <c r="K7" s="39"/>
+      <c r="L7" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M7" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="H8" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="K8" s="33"/>
-      <c r="L8" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="M8" s="32" t="s">
+      <c r="C8" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="N8" s="5" t="s">
-        <v>76</v>
+      <c r="D8" s="45" t="s">
+        <v>81</v>
+      </c>
+      <c r="E8" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="G8" s="45" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="J8" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="K8" s="39"/>
+      <c r="L8" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="M8" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B9" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="35"/>
+      <c r="B9" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="41"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="8">
         <f>'Detailed Cap Table'!C4</f>
         <v>3600000</v>
       </c>
-      <c r="E10" s="1"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="L10" s="27">
+      <c r="E10" s="2"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="L10" s="32">
         <f>C10+E10+H10+J10</f>
         <v>3600000</v>
       </c>
-      <c r="M10" s="41">
+      <c r="M10" s="47">
         <f>L10/$L$21</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="N10" s="38">
+      <c r="N10" s="44">
         <v>50000000</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="8">
         <f>'Detailed Cap Table'!C5</f>
         <v>3600000</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="L11" s="27">
+      <c r="E11" s="2"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="L11" s="32">
         <f>C11+E11+H11+J11</f>
         <v>3600000</v>
       </c>
-      <c r="M11" s="41">
+      <c r="M11" s="47">
         <f>L11/$L$21</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="6">
+      <c r="B12" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="8">
         <f>SUM('Detailed Cap Table'!C6:'Detailed Cap Table'!C10)</f>
         <v>1429687</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="L12" s="27">
+      <c r="E12" s="2"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="L12" s="32">
         <f>C12+E12+H12+J12</f>
         <v>1429687</v>
       </c>
-      <c r="M12" s="41">
+      <c r="M12" s="47">
         <f>L12/$L$21</f>
         <v>0.14678114954390861</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B13" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="6">
+      <c r="B13" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="8">
         <f>'Detailed Cap Table'!D9+'Detailed Cap Table'!D11+'Detailed Cap Table'!D14+'Detailed Cap Table'!D15+'Detailed Cap Table'!D16+'Detailed Cap Table'!E12+'Detailed Cap Table'!E13+'Detailed Cap Table'!E17+'Detailed Cap Table'!E18+'Detailed Cap Table'!F19+'Detailed Cap Table'!F20</f>
         <v>1045471</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="L13" s="27">
+      <c r="E13" s="2"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="L13" s="32">
         <f>C13+E13+H13+J13</f>
         <v>1045471</v>
       </c>
-      <c r="M13" s="41">
+      <c r="M13" s="47">
         <f>L13/$L$21</f>
         <v>0.10733498674522443</v>
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B14" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="6">
+      <c r="B14" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="8">
         <f>'Detailed Cap Table'!D21</f>
         <v>65105</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="L14" s="27">
+      <c r="E14" s="2"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="L14" s="32">
         <f>C14+E14+H14+J14</f>
         <v>65105</v>
       </c>
-      <c r="M14" s="41">
+      <c r="M14" s="47">
         <f>L14/$L$21</f>
         <v>6.6841110963841528E-3</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B15" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C15" s="43">
+      <c r="B15" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="49">
         <f>SUM(C10:C14)</f>
         <v>9740263</v>
       </c>
@@ -2874,173 +2988,922 @@
         <f>SUM(D10:D14)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <f>SUM(E10:E14)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="13">
         <f>SUM(G10:G14)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <f>SUM(H10:H14)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="43">
+      <c r="J15" s="49">
         <f>SUM(J10:J14)</f>
         <v>0</v>
       </c>
-      <c r="L15" s="43">
+      <c r="L15" s="49">
         <f>SUM(L10:L14)</f>
         <v>9740263</v>
       </c>
-      <c r="M15" s="44">
+      <c r="M15" s="50">
         <f>L15/$L$21</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B16" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="42"/>
+      <c r="B16" s="35" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="48"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="G17" s="36">
+      <c r="C17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="G17" s="42">
         <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
         <v>8000000</v>
       </c>
-      <c r="H17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="L17" s="27">
+      <c r="H17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="L17" s="32">
         <f>C17+E17+H17+J17</f>
         <v>0</v>
       </c>
-      <c r="M17" s="41">
+      <c r="M17" s="47">
         <f>L17/$L$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B18" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="G18" s="36">
+      <c r="B18" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="G18" s="42">
         <f>'SAFE Investments'!C27-G17</f>
         <v>1825000</v>
       </c>
-      <c r="H18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="L18" s="27">
+      <c r="H18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="L18" s="32">
         <f>C18+E18+H18+J18</f>
         <v>0</v>
       </c>
-      <c r="M18" s="41">
+      <c r="M18" s="47">
         <f>L18/$L$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B19" s="13"/>
-      <c r="C19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="42"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="48"/>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B20" s="13"/>
-      <c r="C20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="42"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="48"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B21" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" s="45">
+      <c r="B21" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="51">
         <f>C15+SUM(C17:C18)</f>
         <v>9740263</v>
       </c>
-      <c r="D21" s="31">
+      <c r="D21" s="36">
         <f>SUM(D10:D20)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="45">
+      <c r="E21" s="51">
         <f>SUM(E10:E20)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="46">
+      <c r="G21" s="52">
         <f>SUM(G10:G20)</f>
         <v>9825000</v>
       </c>
-      <c r="H21" s="45">
+      <c r="H21" s="51">
         <f>SUM(H10:H20)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="43">
+      <c r="J21" s="49">
         <f>J14</f>
         <v>0</v>
       </c>
-      <c r="L21" s="45">
+      <c r="L21" s="51">
         <f>SUM(L17:L20)+L15</f>
         <v>9740263</v>
       </c>
-      <c r="M21" s="47">
+      <c r="M21" s="53">
         <f>SUM(M17:M18)+M15</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="13"/>
-      <c r="M22" s="15"/>
+      <c r="B22" s="17"/>
+      <c r="M22" s="19"/>
     </row>
     <row r="23" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="M23" s="19"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B24" s="17"/>
+      <c r="M24" s="19"/>
+    </row>
+    <row r="25" spans="2:13" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="40" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="54">
+        <v>50000000</v>
+      </c>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="20"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD74E04D-AD22-AD44-80FE-B463A917015D}">
+  <dimension ref="B1:T34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="15.5" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="0.5" customWidth="1"/>
+    <col min="14" max="14" width="15.5" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="0.5" customWidth="1"/>
+    <col min="17" max="17" width="13.83203125" customWidth="1"/>
+    <col min="18" max="18" width="0.5" customWidth="1"/>
+    <col min="19" max="19" width="14.33203125" customWidth="1"/>
+    <col min="20" max="20" width="9.33203125" customWidth="1"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1"/>
+    <col min="22" max="22" width="15.5" customWidth="1"/>
+    <col min="23" max="23" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B1" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+    </row>
+    <row r="2" spans="2:20" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+    </row>
+    <row r="3" spans="2:20" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+    </row>
+    <row r="4" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="43"/>
+      <c r="G4" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="43"/>
+      <c r="L4" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" s="43"/>
+      <c r="Q4" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="S4" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="T4" s="43"/>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C5" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="L5" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="N5" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q5" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="S5" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="T5" s="25" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="I6" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="J6" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="O6" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q6" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="S6" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="T6" s="37" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B7" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="41"/>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B8" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="8">
+        <f>'Series Seed'!C10</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="38"/>
+      <c r="E8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="N8" s="38"/>
+      <c r="O8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="S8" s="2">
+        <f>C8+E8+G8+J8+L8+O8+Q8</f>
+        <v>3600000</v>
+      </c>
+      <c r="T8" s="48">
+        <f ca="1">S8/$S$21</f>
+        <v>0.18689423878262076</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B9" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="8">
+        <f>'Series Seed'!C11</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="38"/>
+      <c r="E9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="N9" s="38"/>
+      <c r="O9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="S9" s="2">
+        <f>C9+E9+G9+J9+L9+O9+Q9</f>
+        <v>3600000</v>
+      </c>
+      <c r="T9" s="48">
+        <f ca="1">S9/$S$21</f>
+        <v>0.18689423878262076</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B10" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="8">
+        <f>'Series Seed'!C12</f>
+        <v>1429687</v>
+      </c>
+      <c r="D10" s="38"/>
+      <c r="E10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="N10" s="38"/>
+      <c r="O10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="S10" s="2">
+        <f>C10+E10+G10+J10+L10+O10+Q10</f>
+        <v>1429687</v>
+      </c>
+      <c r="T10" s="48">
+        <f ca="1">S10/$S$21</f>
+        <v>7.4222295434002425E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B11" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="8">
+        <f>'Series Seed'!C13</f>
+        <v>1045471</v>
+      </c>
+      <c r="D11" s="38"/>
+      <c r="E11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="N11" s="38"/>
+      <c r="O11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="S11" s="2">
+        <f>C11+E11+G11+J11+L11+O11+Q11</f>
+        <v>1045471</v>
+      </c>
+      <c r="T11" s="48">
+        <f ca="1">S11/$S$21</f>
+        <v>5.4275696309529255E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B12" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="8">
+        <f>'Series Seed'!C14</f>
+        <v>65105</v>
+      </c>
+      <c r="D12" s="38"/>
+      <c r="E12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="N12" s="38"/>
+      <c r="O12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="S12" s="2">
+        <f>C12+E12+G12+J12+L12+O12+Q12</f>
+        <v>65105</v>
+      </c>
+      <c r="T12" s="48">
+        <f ca="1">S12/$S$21</f>
+        <v>3.379930393317368E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="17"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="N13" s="38"/>
+      <c r="O13" s="2"/>
+      <c r="Q13" s="2">
+        <f ca="1">IFERROR(ROUND(((O21+C21+E21+G21+J21+L21)/(1-C33))*C33-C12,0),0)</f>
+        <v>1867629</v>
+      </c>
+      <c r="S13" s="2">
+        <f ca="1">C13+E13+G13+J13+L13+O13+Q13</f>
+        <v>1867629</v>
+      </c>
+      <c r="T13" s="48">
+        <f ca="1">S13/$S$21</f>
+        <v>9.6958083412040902E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B14" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="49">
+        <f>SUM(C8:C13)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D14" s="38">
+        <f>SUM(D8:D13)</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <f>SUM(E8:E13)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="49">
+        <f>SUM(G8:G13)</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="38"/>
+      <c r="J14" s="2">
+        <f>SUM(J8:J13)</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="49">
+        <f>SUM(L8:L13)</f>
+        <v>0</v>
+      </c>
+      <c r="N14" s="38"/>
+      <c r="O14" s="2">
+        <f>SUM(O8:O13)</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="49">
+        <f ca="1">SUM(Q8:Q13)</f>
+        <v>1867629</v>
+      </c>
+      <c r="S14" s="49">
+        <f ca="1">SUM(S8:S13)</f>
+        <v>11607892</v>
+      </c>
+      <c r="T14" s="50">
+        <f ca="1">S14/$S$21</f>
+        <v>0.60262448311413153</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B15" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="N15" s="38"/>
+      <c r="O15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="48"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B16" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="55">
+        <f>'Series Seed'!G17</f>
+        <v>8000000</v>
+      </c>
+      <c r="E16" s="2">
+        <f ca="1">IFERROR(ROUND(D16/$E$23,0),0)</f>
+        <v>2311471</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="N16" s="57">
+        <v>5000000</v>
+      </c>
+      <c r="O16" s="2">
+        <f ca="1">IFERROR(ROUND(N16/$O$23,0),0)</f>
+        <v>1203891</v>
+      </c>
+      <c r="Q16" s="2"/>
+      <c r="S16" s="2">
+        <f ca="1">E16+C16+J16+O16</f>
+        <v>3515362</v>
+      </c>
+      <c r="T16" s="48">
+        <f ca="1">S16/$S$21</f>
+        <v>0.18250025139870871</v>
+      </c>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B17" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="N17" s="57">
+        <v>12000000</v>
+      </c>
+      <c r="O17" s="2">
+        <f ca="1">IFERROR(ROUND(N17/$O$23,0),0)</f>
+        <v>2889338</v>
+      </c>
+      <c r="Q17" s="2"/>
+      <c r="S17" s="2">
+        <f ca="1">E17+C17+J17+O17</f>
+        <v>2889338</v>
+      </c>
+      <c r="T17" s="48">
+        <f ca="1">S17/$S$21</f>
+        <v>0.15000017391547221</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B18" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="I18" s="38"/>
+      <c r="J18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="N18" s="57">
+        <v>3000000</v>
+      </c>
+      <c r="O18" s="2">
+        <f ca="1">IFERROR(ROUND(N18/$O$23,0),0)</f>
+        <v>722335</v>
+      </c>
+      <c r="Q18" s="2"/>
+      <c r="S18" s="2">
+        <f ca="1">E18+C18+J18+O18</f>
+        <v>722335</v>
+      </c>
+      <c r="T18" s="48">
+        <f ca="1">S18/$S$21</f>
+        <v>3.7500069436401218E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B19" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="55">
+        <f>'Series Seed'!G18</f>
+        <v>1825000</v>
+      </c>
+      <c r="E19" s="2">
+        <f ca="1">IFERROR(ROUND(D19/$E$23,0),0)</f>
+        <v>527304</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="I19" s="38"/>
+      <c r="J19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="N19" s="38"/>
+      <c r="O19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="S19" s="2">
+        <f ca="1">E19+C19+J19+O19</f>
+        <v>527304</v>
+      </c>
+      <c r="T19" s="48">
+        <f ca="1">S19/$S$21</f>
+        <v>2.7375022135286406E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B20" s="17"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="I20" s="38"/>
+      <c r="J20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="N20" s="38"/>
+      <c r="O20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="48"/>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B21" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="51">
+        <f>C14+SUM(C16:C19)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D21" s="59">
+        <f>SUM(D8:D19)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E21" s="51">
+        <f ca="1">SUM(E8:E19)</f>
+        <v>2838775</v>
+      </c>
+      <c r="G21" s="49">
+        <f>G13</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="59">
+        <f>SUM(I16:I20)</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="51">
+        <f>SUM(J16:J20)</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="49">
+        <f>L13</f>
+        <v>0</v>
+      </c>
+      <c r="N21" s="59">
+        <f>C30</f>
+        <v>20000000</v>
+      </c>
+      <c r="O21" s="51">
+        <f ca="1">SUM(O16:O20)</f>
+        <v>4815564</v>
+      </c>
+      <c r="Q21" s="49">
+        <f ca="1">Q13</f>
+        <v>1867629</v>
+      </c>
+      <c r="S21" s="51">
+        <f ca="1">SUM(S16:S20)+S14</f>
+        <v>19262231</v>
+      </c>
+      <c r="T21" s="53">
+        <f ca="1">SUM(T16:T19)+T14</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="17"/>
+      <c r="T22" s="19"/>
+    </row>
+    <row r="23" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" s="60">
+        <f ca="1">IFERROR(ROUND(50000000/(C21+E21+G21+Q13),4),0)</f>
+        <v>3.4609999999999999</v>
+      </c>
+      <c r="O23" s="60">
+        <f ca="1">IFERROR(ROUND(O24/(L21+J21+G21+E21+C21+Q13),4),0)</f>
+        <v>4.1532</v>
+      </c>
+      <c r="T23" s="19"/>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B24" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="O24" s="13">
+        <f>O25-N21</f>
+        <v>60000000</v>
+      </c>
+      <c r="T24" s="19"/>
+    </row>
+    <row r="25" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="16">
+        <f>50000000</f>
+        <v>50000000</v>
+      </c>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="16">
+        <f>C30/C31</f>
+        <v>80000000</v>
+      </c>
+      <c r="P25" s="15"/>
+      <c r="Q25" s="15"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="15"/>
+      <c r="T25" s="20"/>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B27" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="M23" s="15"/>
-    </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B24" s="13"/>
-      <c r="M24" s="15"/>
-    </row>
-    <row r="25" spans="2:13" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="48">
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="1">
+        <f>O24/E25-1</f>
+        <v>0.19999999999999996</v>
+      </c>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="57">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="9">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>85</v>
+      </c>
+      <c r="C32" s="56">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>89</v>
+      </c>
+      <c r="C33" s="58">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" s="57">
         <v>50000000</v>
       </c>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Sheet 5: Series B with pro-rata follow-ons and option pool
</commit_message>
<xml_diff>
--- a/runs/20260414-171016/models/model.xlsx
+++ b/runs/20260414-171016/models/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2419F7D4-6A8B-3C49-8C12-A100E19F55BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D901AAF0-B279-1641-B1E4-FC8CA3E5508A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="143" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="SAFE Investments" sheetId="145" r:id="rId3"/>
     <sheet name="Series Seed" sheetId="146" r:id="rId4"/>
     <sheet name="Series A" sheetId="147" r:id="rId5"/>
+    <sheet name="Series B" sheetId="148" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="104">
   <si>
     <t>Total</t>
   </si>
@@ -264,6 +265,15 @@
     <t>Total Raised</t>
   </si>
   <si>
+    <t>Series B</t>
+  </si>
+  <si>
+    <t>Pre B</t>
+  </si>
+  <si>
+    <t>Series B Assumptions:</t>
+  </si>
+  <si>
     <t>% Ownership</t>
   </si>
   <si>
@@ -282,6 +292,9 @@
     <t>Other SAFE Investors</t>
   </si>
   <si>
+    <t>Other Series B Investors</t>
+  </si>
+  <si>
     <t>Invested</t>
   </si>
   <si>
@@ -303,6 +316,9 @@
     <t>SAFE Conversion</t>
   </si>
   <si>
+    <t>% New Money</t>
+  </si>
+  <si>
     <t>SAFE Valuation Cap</t>
   </si>
   <si>
@@ -325,6 +341,15 @@
   </si>
   <si>
     <t>SERIES A ROUND</t>
+  </si>
+  <si>
+    <t>SERIES B ROUND</t>
+  </si>
+  <si>
+    <t>Post B</t>
+  </si>
+  <si>
+    <t>Option Pool Gross %</t>
   </si>
 </sst>
 </file>
@@ -1049,7 +1074,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1068,6 +1093,7 @@
     </xf>
     <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="21" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1075,6 +1101,7 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
@@ -1153,6 +1180,7 @@
     <xf numFmtId="9" fontId="21" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="175" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1596,7 +1624,7 @@
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="29" t="s">
         <v>1</v>
       </c>
       <c r="I2" s="5"/>
@@ -1609,25 +1637,25 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="G3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="H3" s="29" t="s">
         <v>7</v>
       </c>
       <c r="I3" s="5"/>
@@ -1640,20 +1668,20 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="28">
+      <c r="C4" s="30">
         <v>3600000</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28">
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="29">
+      <c r="H4" s="31">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
@@ -1667,20 +1695,20 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="28">
+      <c r="C5" s="30">
         <v>3600000</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28">
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="29">
+      <c r="H5" s="31">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
@@ -1694,20 +1722,20 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="30">
         <v>222187</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28">
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="29">
+      <c r="H6" s="31">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
@@ -1721,20 +1749,20 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="30">
         <v>592500</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28">
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="29">
+      <c r="H7" s="31">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
@@ -1748,20 +1776,20 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="28">
+      <c r="C8" s="30">
         <v>592500</v>
       </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28">
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="29">
+      <c r="H8" s="31">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
@@ -1775,22 +1803,22 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="30">
         <v>13500</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="30">
         <v>98900</v>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28">
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="29">
+      <c r="H9" s="31">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
@@ -1804,20 +1832,20 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="30">
         <v>9000</v>
       </c>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28">
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="29">
+      <c r="H10" s="31">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
@@ -1831,20 +1859,20 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28">
+      <c r="C11" s="30"/>
+      <c r="D11" s="30">
         <v>95000</v>
       </c>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28">
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="29">
+      <c r="H11" s="31">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
@@ -1858,20 +1886,20 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28">
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30">
         <v>25000</v>
       </c>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28">
+      <c r="F12" s="30"/>
+      <c r="G12" s="30">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="29">
+      <c r="H12" s="31">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
@@ -1885,20 +1913,20 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28">
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30">
         <v>41562</v>
       </c>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28">
+      <c r="F13" s="30"/>
+      <c r="G13" s="30">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="29">
+      <c r="H13" s="31">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
@@ -1912,20 +1940,20 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28">
+      <c r="C14" s="30"/>
+      <c r="D14" s="30">
         <v>285000</v>
       </c>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28">
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="29">
+      <c r="H14" s="31">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
@@ -1939,20 +1967,20 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28">
+      <c r="C15" s="30"/>
+      <c r="D15" s="30">
         <v>50000</v>
       </c>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28">
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="29">
+      <c r="H15" s="31">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
@@ -1966,20 +1994,20 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28">
+      <c r="C16" s="30"/>
+      <c r="D16" s="30">
         <v>285000</v>
       </c>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28">
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="29">
+      <c r="H16" s="31">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
@@ -1993,20 +2021,20 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28">
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30">
         <v>96186</v>
       </c>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28">
+      <c r="F17" s="30"/>
+      <c r="G17" s="30">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="29">
+      <c r="H17" s="31">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
@@ -2020,20 +2048,20 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="5"/>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28">
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30">
         <v>48095</v>
       </c>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28">
+      <c r="F18" s="30"/>
+      <c r="G18" s="30">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="29">
+      <c r="H18" s="31">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
@@ -2047,20 +2075,20 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="5"/>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28">
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30">
         <v>12395</v>
       </c>
-      <c r="G19" s="28">
+      <c r="G19" s="30">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="29">
+      <c r="H19" s="31">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
@@ -2074,20 +2102,20 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28">
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30">
         <v>8333</v>
       </c>
-      <c r="G20" s="28">
+      <c r="G20" s="30">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="29">
+      <c r="H20" s="31">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
@@ -2101,20 +2129,20 @@
     </row>
     <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5"/>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28">
+      <c r="C21" s="30"/>
+      <c r="D21" s="30">
         <v>65105</v>
       </c>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28">
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="29">
+      <c r="H21" s="31">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
@@ -2145,26 +2173,26 @@
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5"/>
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="28">
+      <c r="C23" s="30">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="28">
+      <c r="D23" s="30">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="28">
+      <c r="E23" s="30">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="28">
+      <c r="F23" s="30">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="28">
+      <c r="G23" s="30">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
@@ -2223,14 +2251,14 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="32" t="s">
         <v>26</v>
       </c>
       <c r="D3" s="5"/>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="29" t="s">
         <v>27</v>
       </c>
       <c r="F3" s="5"/>
@@ -2242,14 +2270,14 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="31">
+      <c r="C4" s="33">
         <v>25000</v>
       </c>
       <c r="D4" s="5"/>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="28" t="s">
         <v>28</v>
       </c>
       <c r="F4" s="5"/>
@@ -2261,14 +2289,14 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="33">
         <v>25000</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="26"/>
+      <c r="E5" s="28"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
@@ -2278,14 +2306,14 @@
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="33">
         <v>137170.75</v>
       </c>
       <c r="D6" s="5"/>
-      <c r="E6" s="26"/>
+      <c r="E6" s="28"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
@@ -2295,14 +2323,14 @@
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="33">
         <v>3846829.25</v>
       </c>
       <c r="D7" s="5"/>
-      <c r="E7" s="26"/>
+      <c r="E7" s="28"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
@@ -2312,15 +2340,15 @@
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="33">
         <v>16566</v>
       </c>
       <c r="D8" s="5"/>
-      <c r="E8" s="26" t="s">
-        <v>83</v>
+      <c r="E8" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
@@ -2331,14 +2359,14 @@
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="33">
         <v>250000</v>
       </c>
       <c r="D9" s="5"/>
-      <c r="E9" s="26"/>
+      <c r="E9" s="28"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
@@ -2348,14 +2376,14 @@
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="33">
         <v>100000</v>
       </c>
       <c r="D10" s="5"/>
-      <c r="E10" s="26"/>
+      <c r="E10" s="28"/>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
@@ -2365,14 +2393,14 @@
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="33">
         <v>300000</v>
       </c>
       <c r="D11" s="5"/>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="28" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="5"/>
@@ -2384,14 +2412,14 @@
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="33">
         <v>37500</v>
       </c>
       <c r="D12" s="5"/>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="28" t="s">
         <v>36</v>
       </c>
       <c r="F12" s="5"/>
@@ -2403,14 +2431,14 @@
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="33">
         <v>250000</v>
       </c>
       <c r="D13" s="5"/>
-      <c r="E13" s="26"/>
+      <c r="E13" s="28"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
@@ -2420,14 +2448,14 @@
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="33">
         <v>100000</v>
       </c>
       <c r="D14" s="5"/>
-      <c r="E14" s="26"/>
+      <c r="E14" s="28"/>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
@@ -2437,15 +2465,15 @@
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="33">
         <v>41164</v>
       </c>
       <c r="D15" s="5"/>
-      <c r="E15" s="26" t="s">
-        <v>83</v>
+      <c r="E15" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
@@ -2456,15 +2484,15 @@
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="33">
         <v>2328778</v>
       </c>
       <c r="D16" s="5"/>
-      <c r="E16" s="26" t="s">
-        <v>83</v>
+      <c r="E16" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
@@ -2475,14 +2503,14 @@
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="31">
+      <c r="C17" s="33">
         <v>1506000</v>
       </c>
       <c r="D17" s="5"/>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="28" t="s">
         <v>42</v>
       </c>
       <c r="F17" s="5"/>
@@ -2494,14 +2522,14 @@
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="5"/>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="33">
         <v>50000</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="26"/>
+      <c r="E18" s="28"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
@@ -2511,14 +2539,14 @@
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5"/>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="31">
+      <c r="C19" s="33">
         <v>212500</v>
       </c>
       <c r="D19" s="5"/>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="28" t="s">
         <v>36</v>
       </c>
       <c r="F19" s="5"/>
@@ -2530,14 +2558,14 @@
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="31">
+      <c r="C20" s="33">
         <v>25000</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="E20" s="26"/>
+      <c r="E20" s="28"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
@@ -2547,15 +2575,15 @@
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5"/>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="31">
+      <c r="C21" s="33">
         <v>61746</v>
       </c>
       <c r="D21" s="5"/>
-      <c r="E21" s="26" t="s">
-        <v>83</v>
+      <c r="E21" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
@@ -2566,14 +2594,14 @@
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="5"/>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="31">
+      <c r="C22" s="33">
         <v>100000</v>
       </c>
       <c r="D22" s="5"/>
-      <c r="E22" s="26"/>
+      <c r="E22" s="28"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
@@ -2583,14 +2611,14 @@
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5"/>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="31">
+      <c r="C23" s="33">
         <v>100000</v>
       </c>
       <c r="D23" s="5"/>
-      <c r="E23" s="26"/>
+      <c r="E23" s="28"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
@@ -2600,15 +2628,15 @@
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="5"/>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="33">
         <v>61746</v>
       </c>
       <c r="D24" s="5"/>
-      <c r="E24" s="26" t="s">
-        <v>83</v>
+      <c r="E24" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
@@ -2619,14 +2647,14 @@
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="5"/>
-      <c r="B25" s="26" t="s">
+      <c r="B25" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="33">
         <v>250000</v>
       </c>
       <c r="D25" s="5"/>
-      <c r="E25" s="26" t="s">
+      <c r="E25" s="28" t="s">
         <v>51</v>
       </c>
       <c r="F25" s="5"/>
@@ -2651,10 +2679,10 @@
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="30">
+      <c r="C27" s="32">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
@@ -2694,182 +2722,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="12"/>
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="11"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="12"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="11"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="12"/>
     </row>
     <row r="4" spans="2:14" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="11"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13"/>
+      <c r="M4" s="13"/>
+      <c r="N4" s="12"/>
     </row>
     <row r="5" spans="2:14" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="12"/>
     </row>
     <row r="6" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="43"/>
-      <c r="G6" s="21" t="s">
+      <c r="D6" s="23"/>
+      <c r="E6" s="45"/>
+      <c r="G6" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="43"/>
-      <c r="J6" s="21" t="s">
+      <c r="H6" s="45"/>
+      <c r="J6" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="17"/>
-      <c r="L6" s="21" t="s">
+      <c r="K6" s="19"/>
+      <c r="L6" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="M6" s="43"/>
+      <c r="M6" s="45"/>
       <c r="N6" s="7" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="G7" s="46" t="s">
+      <c r="G7" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="25" t="s">
+      <c r="H7" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="J7" s="24" t="s">
+      <c r="J7" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="K7" s="39"/>
-      <c r="L7" s="21" t="s">
+      <c r="K7" s="41"/>
+      <c r="L7" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="M7" s="25" t="s">
-        <v>84</v>
+      <c r="M7" s="27" t="s">
+        <v>88</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="45" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" s="37" t="s">
+      <c r="D8" s="47" t="s">
+        <v>85</v>
+      </c>
+      <c r="E8" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="45" t="s">
-        <v>81</v>
-      </c>
-      <c r="H8" s="37" t="s">
+      <c r="G8" s="47" t="s">
+        <v>85</v>
+      </c>
+      <c r="H8" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="J8" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="K8" s="39"/>
-      <c r="L8" s="23" t="s">
+      <c r="J8" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="K8" s="41"/>
+      <c r="L8" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="M8" s="37" t="s">
+      <c r="M8" s="39" t="s">
         <v>64</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="41"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="43"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="36" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="8">
@@ -2877,23 +2905,23 @@
         <v>3600000</v>
       </c>
       <c r="E10" s="2"/>
-      <c r="G10" s="13"/>
+      <c r="G10" s="15"/>
       <c r="H10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="L10" s="32">
+      <c r="L10" s="34">
         <f>C10+E10+H10+J10</f>
         <v>3600000</v>
       </c>
-      <c r="M10" s="47">
+      <c r="M10" s="49">
         <f>L10/$L$21</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="N10" s="44">
+      <c r="N10" s="46">
         <v>50000000</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="36" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="8">
@@ -2901,86 +2929,86 @@
         <v>3600000</v>
       </c>
       <c r="E11" s="2"/>
-      <c r="G11" s="13"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="L11" s="32">
+      <c r="L11" s="34">
         <f>C11+E11+H11+J11</f>
         <v>3600000</v>
       </c>
-      <c r="M11" s="47">
+      <c r="M11" s="49">
         <f>L11/$L$21</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="34" t="s">
-        <v>77</v>
+      <c r="B12" s="36" t="s">
+        <v>80</v>
       </c>
       <c r="C12" s="8">
         <f>SUM('Detailed Cap Table'!C6:'Detailed Cap Table'!C10)</f>
         <v>1429687</v>
       </c>
       <c r="E12" s="2"/>
-      <c r="G12" s="13"/>
+      <c r="G12" s="15"/>
       <c r="H12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="L12" s="32">
+      <c r="L12" s="34">
         <f>C12+E12+H12+J12</f>
         <v>1429687</v>
       </c>
-      <c r="M12" s="47">
+      <c r="M12" s="49">
         <f>L12/$L$21</f>
         <v>0.14678114954390861</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B13" s="34" t="s">
-        <v>78</v>
+      <c r="B13" s="36" t="s">
+        <v>81</v>
       </c>
       <c r="C13" s="8">
         <f>'Detailed Cap Table'!D9+'Detailed Cap Table'!D11+'Detailed Cap Table'!D14+'Detailed Cap Table'!D15+'Detailed Cap Table'!D16+'Detailed Cap Table'!E12+'Detailed Cap Table'!E13+'Detailed Cap Table'!E17+'Detailed Cap Table'!E18+'Detailed Cap Table'!F19+'Detailed Cap Table'!F20</f>
         <v>1045471</v>
       </c>
       <c r="E13" s="2"/>
-      <c r="G13" s="13"/>
+      <c r="G13" s="15"/>
       <c r="H13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="L13" s="32">
+      <c r="L13" s="34">
         <f>C13+E13+H13+J13</f>
         <v>1045471</v>
       </c>
-      <c r="M13" s="47">
+      <c r="M13" s="49">
         <f>L13/$L$21</f>
         <v>0.10733498674522443</v>
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B14" s="34" t="s">
-        <v>79</v>
+      <c r="B14" s="36" t="s">
+        <v>82</v>
       </c>
       <c r="C14" s="8">
         <f>'Detailed Cap Table'!D21</f>
         <v>65105</v>
       </c>
       <c r="E14" s="2"/>
-      <c r="G14" s="13"/>
+      <c r="G14" s="15"/>
       <c r="H14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="L14" s="32">
+      <c r="L14" s="34">
         <f>C14+E14+H14+J14</f>
         <v>65105</v>
       </c>
-      <c r="M14" s="47">
+      <c r="M14" s="49">
         <f>L14/$L$21</f>
         <v>6.6841110963841528E-3</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="49">
+      <c r="C15" s="51">
         <f>SUM(C10:C14)</f>
         <v>9740263</v>
       </c>
@@ -2992,7 +3020,7 @@
         <f>SUM(E10:E14)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="13">
+      <c r="G15" s="15">
         <f>SUM(G10:G14)</f>
         <v>0</v>
       </c>
@@ -3000,161 +3028,161 @@
         <f>SUM(H10:H14)</f>
         <v>0</v>
       </c>
-      <c r="J15" s="49">
+      <c r="J15" s="51">
         <f>SUM(J10:J14)</f>
         <v>0</v>
       </c>
-      <c r="L15" s="49">
+      <c r="L15" s="51">
         <f>SUM(L10:L14)</f>
         <v>9740263</v>
       </c>
-      <c r="M15" s="50">
+      <c r="M15" s="52">
         <f>L15/$L$21</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B16" s="35" t="s">
-        <v>93</v>
+      <c r="B16" s="37" t="s">
+        <v>98</v>
       </c>
       <c r="C16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="G16" s="13"/>
+      <c r="G16" s="15"/>
       <c r="H16" s="2"/>
       <c r="J16" s="2"/>
       <c r="L16" s="2"/>
-      <c r="M16" s="48"/>
+      <c r="M16" s="50"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="36" t="s">
         <v>42</v>
       </c>
       <c r="C17" s="2"/>
       <c r="E17" s="2"/>
-      <c r="G17" s="42">
+      <c r="G17" s="44">
         <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
         <v>8000000</v>
       </c>
       <c r="H17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="L17" s="32">
+      <c r="L17" s="34">
         <f>C17+E17+H17+J17</f>
         <v>0</v>
       </c>
-      <c r="M17" s="47">
+      <c r="M17" s="49">
         <f>L17/$L$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B18" s="34" t="s">
-        <v>80</v>
+      <c r="B18" s="36" t="s">
+        <v>83</v>
       </c>
       <c r="C18" s="2"/>
       <c r="E18" s="2"/>
-      <c r="G18" s="42">
+      <c r="G18" s="44">
         <f>'SAFE Investments'!C27-G17</f>
         <v>1825000</v>
       </c>
       <c r="H18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="L18" s="32">
+      <c r="L18" s="34">
         <f>C18+E18+H18+J18</f>
         <v>0</v>
       </c>
-      <c r="M18" s="47">
+      <c r="M18" s="49">
         <f>L18/$L$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B19" s="17"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="G19" s="13"/>
+      <c r="G19" s="15"/>
       <c r="H19" s="2"/>
       <c r="J19" s="2"/>
       <c r="L19" s="2"/>
-      <c r="M19" s="48"/>
+      <c r="M19" s="50"/>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B20" s="17"/>
+      <c r="B20" s="19"/>
       <c r="C20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="G20" s="13"/>
+      <c r="G20" s="15"/>
       <c r="H20" s="2"/>
       <c r="J20" s="2"/>
       <c r="L20" s="2"/>
-      <c r="M20" s="48"/>
+      <c r="M20" s="50"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="51">
+      <c r="C21" s="53">
         <f>C15+SUM(C17:C18)</f>
         <v>9740263</v>
       </c>
-      <c r="D21" s="36">
+      <c r="D21" s="38">
         <f>SUM(D10:D20)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="51">
+      <c r="E21" s="53">
         <f>SUM(E10:E20)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="52">
+      <c r="G21" s="54">
         <f>SUM(G10:G20)</f>
         <v>9825000</v>
       </c>
-      <c r="H21" s="51">
+      <c r="H21" s="53">
         <f>SUM(H10:H20)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="49">
+      <c r="J21" s="51">
         <f>J14</f>
         <v>0</v>
       </c>
-      <c r="L21" s="51">
+      <c r="L21" s="53">
         <f>SUM(L17:L20)+L15</f>
         <v>9740263</v>
       </c>
-      <c r="M21" s="53">
+      <c r="M21" s="55">
         <f>SUM(M17:M18)+M15</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="17"/>
-      <c r="M22" s="19"/>
+      <c r="B22" s="19"/>
+      <c r="M22" s="21"/>
     </row>
     <row r="23" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="M23" s="19"/>
+      <c r="B23" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="M23" s="21"/>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B24" s="17"/>
-      <c r="M24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="M24" s="21"/>
     </row>
     <row r="25" spans="2:13" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="40" t="s">
-        <v>94</v>
-      </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="54">
+      <c r="B25" s="42" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="56">
         <v>50000000</v>
       </c>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
-      <c r="M25" s="20"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3192,343 +3220,343 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
     </row>
     <row r="2" spans="2:20" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+    </row>
+    <row r="3" spans="2:20" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+    </row>
+    <row r="4" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="45"/>
+      <c r="G4" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="J4" s="45"/>
+      <c r="L4" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" s="45"/>
+      <c r="Q4" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="S4" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="T4" s="45"/>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C5" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="L5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="N5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="S5" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="T5" s="27" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-    </row>
-    <row r="3" spans="2:20" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-    </row>
-    <row r="4" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="43"/>
-      <c r="G4" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="43"/>
-      <c r="L4" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="N4" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="O4" s="43"/>
-      <c r="Q4" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="S4" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="T4" s="43"/>
-    </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="C5" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="G5" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="J5" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="L5" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="O5" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q5" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="S5" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="T5" s="25" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="23" t="s">
+      <c r="I6" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="J6" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="E6" s="37" t="s">
+      <c r="L6" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="G6" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="I6" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="J6" s="37" t="s">
+      <c r="Q6" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="S6" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="L6" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="N6" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="O6" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q6" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="S6" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="T6" s="37" t="s">
+      <c r="T6" s="39" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="14"/>
-      <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="14"/>
-      <c r="Q7" s="14"/>
-      <c r="R7" s="14"/>
-      <c r="S7" s="14"/>
-      <c r="T7" s="41"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="43"/>
     </row>
     <row r="8" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="36" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="8">
         <f>'Series Seed'!C10</f>
         <v>3600000</v>
       </c>
-      <c r="D8" s="38"/>
+      <c r="D8" s="40"/>
       <c r="E8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="I8" s="38"/>
+      <c r="I8" s="40"/>
       <c r="J8" s="2"/>
       <c r="L8" s="2"/>
-      <c r="N8" s="38"/>
+      <c r="N8" s="40"/>
       <c r="O8" s="2"/>
       <c r="Q8" s="2"/>
       <c r="S8" s="2">
         <f>C8+E8+G8+J8+L8+O8+Q8</f>
         <v>3600000</v>
       </c>
-      <c r="T8" s="48">
+      <c r="T8" s="50">
         <f ca="1">S8/$S$21</f>
         <v>0.18689423878262076</v>
       </c>
     </row>
     <row r="9" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="36" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="8">
         <f>'Series Seed'!C11</f>
         <v>3600000</v>
       </c>
-      <c r="D9" s="38"/>
+      <c r="D9" s="40"/>
       <c r="E9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="I9" s="38"/>
+      <c r="I9" s="40"/>
       <c r="J9" s="2"/>
       <c r="L9" s="2"/>
-      <c r="N9" s="38"/>
+      <c r="N9" s="40"/>
       <c r="O9" s="2"/>
       <c r="Q9" s="2"/>
       <c r="S9" s="2">
         <f>C9+E9+G9+J9+L9+O9+Q9</f>
         <v>3600000</v>
       </c>
-      <c r="T9" s="48">
+      <c r="T9" s="50">
         <f ca="1">S9/$S$21</f>
         <v>0.18689423878262076</v>
       </c>
     </row>
     <row r="10" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B10" s="34" t="s">
-        <v>77</v>
+      <c r="B10" s="36" t="s">
+        <v>80</v>
       </c>
       <c r="C10" s="8">
         <f>'Series Seed'!C12</f>
         <v>1429687</v>
       </c>
-      <c r="D10" s="38"/>
+      <c r="D10" s="40"/>
       <c r="E10" s="2"/>
       <c r="G10" s="2"/>
-      <c r="I10" s="38"/>
+      <c r="I10" s="40"/>
       <c r="J10" s="2"/>
       <c r="L10" s="2"/>
-      <c r="N10" s="38"/>
+      <c r="N10" s="40"/>
       <c r="O10" s="2"/>
       <c r="Q10" s="2"/>
       <c r="S10" s="2">
         <f>C10+E10+G10+J10+L10+O10+Q10</f>
         <v>1429687</v>
       </c>
-      <c r="T10" s="48">
+      <c r="T10" s="50">
         <f ca="1">S10/$S$21</f>
         <v>7.4222295434002425E-2</v>
       </c>
     </row>
     <row r="11" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B11" s="34" t="s">
-        <v>78</v>
+      <c r="B11" s="36" t="s">
+        <v>81</v>
       </c>
       <c r="C11" s="8">
         <f>'Series Seed'!C13</f>
         <v>1045471</v>
       </c>
-      <c r="D11" s="38"/>
+      <c r="D11" s="40"/>
       <c r="E11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="I11" s="38"/>
+      <c r="I11" s="40"/>
       <c r="J11" s="2"/>
       <c r="L11" s="2"/>
-      <c r="N11" s="38"/>
+      <c r="N11" s="40"/>
       <c r="O11" s="2"/>
       <c r="Q11" s="2"/>
       <c r="S11" s="2">
         <f>C11+E11+G11+J11+L11+O11+Q11</f>
         <v>1045471</v>
       </c>
-      <c r="T11" s="48">
+      <c r="T11" s="50">
         <f ca="1">S11/$S$21</f>
         <v>5.4275696309529255E-2</v>
       </c>
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B12" s="34" t="s">
-        <v>79</v>
+      <c r="B12" s="36" t="s">
+        <v>82</v>
       </c>
       <c r="C12" s="8">
         <f>'Series Seed'!C14</f>
         <v>65105</v>
       </c>
-      <c r="D12" s="38"/>
+      <c r="D12" s="40"/>
       <c r="E12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="I12" s="38"/>
+      <c r="I12" s="40"/>
       <c r="J12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="N12" s="38"/>
+      <c r="N12" s="40"/>
       <c r="O12" s="2"/>
       <c r="Q12" s="2"/>
       <c r="S12" s="2">
         <f>C12+E12+G12+J12+L12+O12+Q12</f>
         <v>65105</v>
       </c>
-      <c r="T12" s="48">
+      <c r="T12" s="50">
         <f ca="1">S12/$S$21</f>
         <v>3.379930393317368E-3</v>
       </c>
     </row>
     <row r="13" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="17"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="38"/>
+      <c r="D13" s="40"/>
       <c r="E13" s="2"/>
       <c r="G13" s="2"/>
-      <c r="I13" s="38"/>
+      <c r="I13" s="40"/>
       <c r="J13" s="2"/>
       <c r="L13" s="2"/>
-      <c r="N13" s="38"/>
+      <c r="N13" s="40"/>
       <c r="O13" s="2"/>
       <c r="Q13" s="2">
         <f ca="1">IFERROR(ROUND(((O21+C21+E21+G21+J21+L21)/(1-C33))*C33-C12,0),0)</f>
@@ -3538,20 +3566,20 @@
         <f ca="1">C13+E13+G13+J13+L13+O13+Q13</f>
         <v>1867629</v>
       </c>
-      <c r="T13" s="48">
+      <c r="T13" s="50">
         <f ca="1">S13/$S$21</f>
         <v>9.6958083412040902E-2</v>
       </c>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="49">
+      <c r="C14" s="51">
         <f>SUM(C8:C13)</f>
         <v>9740263</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="40">
         <f>SUM(D8:D13)</f>
         <v>0</v>
       </c>
@@ -3559,60 +3587,60 @@
         <f>SUM(E8:E13)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="49">
+      <c r="G14" s="51">
         <f>SUM(G8:G13)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="40"/>
       <c r="J14" s="2">
         <f>SUM(J8:J13)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="49">
+      <c r="L14" s="51">
         <f>SUM(L8:L13)</f>
         <v>0</v>
       </c>
-      <c r="N14" s="38"/>
+      <c r="N14" s="40"/>
       <c r="O14" s="2">
         <f>SUM(O8:O13)</f>
         <v>0</v>
       </c>
-      <c r="Q14" s="49">
+      <c r="Q14" s="51">
         <f ca="1">SUM(Q8:Q13)</f>
         <v>1867629</v>
       </c>
-      <c r="S14" s="49">
+      <c r="S14" s="51">
         <f ca="1">SUM(S8:S13)</f>
         <v>11607892</v>
       </c>
-      <c r="T14" s="50">
+      <c r="T14" s="52">
         <f ca="1">S14/$S$21</f>
         <v>0.60262448311413153</v>
       </c>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="37" t="s">
         <v>67</v>
       </c>
       <c r="C15" s="2"/>
-      <c r="D15" s="38"/>
+      <c r="D15" s="40"/>
       <c r="E15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="I15" s="38"/>
+      <c r="I15" s="40"/>
       <c r="J15" s="2"/>
       <c r="L15" s="2"/>
-      <c r="N15" s="38"/>
+      <c r="N15" s="40"/>
       <c r="O15" s="2"/>
       <c r="Q15" s="2"/>
       <c r="S15" s="2"/>
-      <c r="T15" s="48"/>
+      <c r="T15" s="50"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="19" t="s">
         <v>42</v>
       </c>
       <c r="C16" s="2"/>
-      <c r="D16" s="55">
+      <c r="D16" s="57">
         <f>'Series Seed'!G17</f>
         <v>8000000</v>
       </c>
@@ -3621,10 +3649,10 @@
         <v>2311471</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="I16" s="38"/>
+      <c r="I16" s="40"/>
       <c r="J16" s="2"/>
       <c r="L16" s="2"/>
-      <c r="N16" s="57">
+      <c r="N16" s="59">
         <v>5000000</v>
       </c>
       <c r="O16" s="2">
@@ -3636,23 +3664,23 @@
         <f ca="1">E16+C16+J16+O16</f>
         <v>3515362</v>
       </c>
-      <c r="T16" s="48">
+      <c r="T16" s="50">
         <f ca="1">S16/$S$21</f>
         <v>0.18250025139870871</v>
       </c>
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="19" t="s">
         <v>68</v>
       </c>
       <c r="C17" s="2"/>
-      <c r="D17" s="38"/>
+      <c r="D17" s="40"/>
       <c r="E17" s="2"/>
       <c r="G17" s="2"/>
-      <c r="I17" s="38"/>
+      <c r="I17" s="40"/>
       <c r="J17" s="2"/>
       <c r="L17" s="2"/>
-      <c r="N17" s="57">
+      <c r="N17" s="59">
         <v>12000000</v>
       </c>
       <c r="O17" s="2">
@@ -3664,23 +3692,23 @@
         <f ca="1">E17+C17+J17+O17</f>
         <v>2889338</v>
       </c>
-      <c r="T17" s="48">
+      <c r="T17" s="50">
         <f ca="1">S17/$S$21</f>
         <v>0.15000017391547221</v>
       </c>
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="19" t="s">
         <v>69</v>
       </c>
       <c r="C18" s="2"/>
-      <c r="D18" s="38"/>
+      <c r="D18" s="40"/>
       <c r="E18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="I18" s="38"/>
+      <c r="I18" s="40"/>
       <c r="J18" s="2"/>
       <c r="L18" s="2"/>
-      <c r="N18" s="57">
+      <c r="N18" s="59">
         <v>3000000</v>
       </c>
       <c r="O18" s="2">
@@ -3692,17 +3720,17 @@
         <f ca="1">E18+C18+J18+O18</f>
         <v>722335</v>
       </c>
-      <c r="T18" s="48">
+      <c r="T18" s="50">
         <f ca="1">S18/$S$21</f>
         <v>3.7500069436401218E-2</v>
       </c>
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B19" s="17" t="s">
-        <v>80</v>
+      <c r="B19" s="19" t="s">
+        <v>83</v>
       </c>
       <c r="C19" s="2"/>
-      <c r="D19" s="55">
+      <c r="D19" s="57">
         <f>'Series Seed'!G18</f>
         <v>1825000</v>
       </c>
@@ -3711,145 +3739,145 @@
         <v>527304</v>
       </c>
       <c r="G19" s="2"/>
-      <c r="I19" s="38"/>
+      <c r="I19" s="40"/>
       <c r="J19" s="2"/>
       <c r="L19" s="2"/>
-      <c r="N19" s="38"/>
+      <c r="N19" s="40"/>
       <c r="O19" s="2"/>
       <c r="Q19" s="2"/>
       <c r="S19" s="2">
         <f ca="1">E19+C19+J19+O19</f>
         <v>527304</v>
       </c>
-      <c r="T19" s="48">
+      <c r="T19" s="50">
         <f ca="1">S19/$S$21</f>
         <v>2.7375022135286406E-2</v>
       </c>
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B20" s="17"/>
+      <c r="B20" s="19"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="38"/>
+      <c r="D20" s="40"/>
       <c r="E20" s="2"/>
       <c r="G20" s="2"/>
-      <c r="I20" s="38"/>
+      <c r="I20" s="40"/>
       <c r="J20" s="2"/>
       <c r="L20" s="2"/>
-      <c r="N20" s="38"/>
+      <c r="N20" s="40"/>
       <c r="O20" s="2"/>
       <c r="Q20" s="2"/>
       <c r="S20" s="2"/>
-      <c r="T20" s="48"/>
+      <c r="T20" s="50"/>
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="51">
+      <c r="C21" s="53">
         <f>C14+SUM(C16:C19)</f>
         <v>9740263</v>
       </c>
-      <c r="D21" s="59">
+      <c r="D21" s="61">
         <f>SUM(D8:D19)</f>
         <v>9825000</v>
       </c>
-      <c r="E21" s="51">
+      <c r="E21" s="53">
         <f ca="1">SUM(E8:E19)</f>
         <v>2838775</v>
       </c>
-      <c r="G21" s="49">
+      <c r="G21" s="51">
         <f>G13</f>
         <v>0</v>
       </c>
-      <c r="I21" s="59">
+      <c r="I21" s="61">
         <f>SUM(I16:I20)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="51">
+      <c r="J21" s="53">
         <f>SUM(J16:J20)</f>
         <v>0</v>
       </c>
-      <c r="L21" s="49">
+      <c r="L21" s="51">
         <f>L13</f>
         <v>0</v>
       </c>
-      <c r="N21" s="59">
+      <c r="N21" s="61">
         <f>C30</f>
         <v>20000000</v>
       </c>
-      <c r="O21" s="51">
+      <c r="O21" s="53">
         <f ca="1">SUM(O16:O20)</f>
         <v>4815564</v>
       </c>
-      <c r="Q21" s="49">
+      <c r="Q21" s="51">
         <f ca="1">Q13</f>
         <v>1867629</v>
       </c>
-      <c r="S21" s="51">
+      <c r="S21" s="53">
         <f ca="1">SUM(S16:S20)+S14</f>
         <v>19262231</v>
       </c>
-      <c r="T21" s="53">
+      <c r="T21" s="55">
         <f ca="1">SUM(T16:T19)+T14</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="17"/>
-      <c r="T22" s="19"/>
+      <c r="B22" s="19"/>
+      <c r="T22" s="21"/>
     </row>
     <row r="23" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="E23" s="60">
+      <c r="B23" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="E23" s="62">
         <f ca="1">IFERROR(ROUND(50000000/(C21+E21+G21+Q13),4),0)</f>
         <v>3.4609999999999999</v>
       </c>
-      <c r="O23" s="60">
+      <c r="O23" s="62">
         <f ca="1">IFERROR(ROUND(O24/(L21+J21+G21+E21+C21+Q13),4),0)</f>
         <v>4.1532</v>
       </c>
-      <c r="T23" s="19"/>
+      <c r="T23" s="21"/>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="O24" s="13">
+      <c r="O24" s="15">
         <f>O25-N21</f>
         <v>60000000</v>
       </c>
-      <c r="T24" s="19"/>
+      <c r="T24" s="21"/>
     </row>
     <row r="25" spans="2:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="40" t="s">
+      <c r="B25" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="16">
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="18">
         <f>50000000</f>
         <v>50000000</v>
       </c>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
-      <c r="N25" s="15"/>
-      <c r="O25" s="16">
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="17"/>
+      <c r="N25" s="17"/>
+      <c r="O25" s="18">
         <f>C30/C31</f>
         <v>80000000</v>
       </c>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="15"/>
-      <c r="S25" s="15"/>
-      <c r="T25" s="20"/>
+      <c r="P25" s="17"/>
+      <c r="Q25" s="17"/>
+      <c r="R25" s="17"/>
+      <c r="S25" s="17"/>
+      <c r="T25" s="22"/>
     </row>
     <row r="27" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B27" s="6" t="s">
@@ -3858,7 +3886,7 @@
     </row>
     <row r="29" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C29" s="1">
         <f>O24/E25-1</f>
@@ -3869,13 +3897,13 @@
       <c r="B30" t="s">
         <v>74</v>
       </c>
-      <c r="C30" s="57">
+      <c r="C30" s="59">
         <v>20000000</v>
       </c>
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C31" s="9">
         <v>0.25</v>
@@ -3883,26 +3911,959 @@
     </row>
     <row r="32" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>85</v>
-      </c>
-      <c r="C32" s="56">
+        <v>89</v>
+      </c>
+      <c r="C32" s="58">
         <v>12000000</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>89</v>
-      </c>
-      <c r="C33" s="58">
+        <v>94</v>
+      </c>
+      <c r="C33" s="60">
         <v>0.1</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
+        <v>93</v>
+      </c>
+      <c r="C34" s="59">
+        <v>50000000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9150141D-2142-2C4D-B443-14315CD35149}">
+  <dimension ref="B1:Y34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="33.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" customWidth="1"/>
+    <col min="5" max="5" width="12.5" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="11.1640625" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="10" max="10" width="15.5" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" customWidth="1"/>
+    <col min="13" max="13" width="0.5" customWidth="1"/>
+    <col min="14" max="14" width="15.5" customWidth="1"/>
+    <col min="15" max="15" width="11.33203125" customWidth="1"/>
+    <col min="16" max="16" width="0.5" customWidth="1"/>
+    <col min="17" max="17" width="11.83203125" customWidth="1"/>
+    <col min="18" max="18" width="0.5" customWidth="1"/>
+    <col min="19" max="19" width="15.5" customWidth="1"/>
+    <col min="20" max="20" width="16.83203125" customWidth="1"/>
+    <col min="21" max="21" width="0.5" customWidth="1"/>
+    <col min="22" max="22" width="11.83203125" customWidth="1"/>
+    <col min="23" max="23" width="0.5" customWidth="1"/>
+    <col min="24" max="24" width="13" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="6.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="13"/>
+      <c r="X1" s="13"/>
+      <c r="Y1" s="13"/>
+    </row>
+    <row r="2" spans="2:25" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+    </row>
+    <row r="3" spans="2:25" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11"/>
+      <c r="W3" s="11"/>
+      <c r="X3" s="11"/>
+      <c r="Y3" s="11"/>
+    </row>
+    <row r="4" spans="2:25" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="27"/>
+      <c r="G4" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="J4" s="27"/>
+      <c r="L4" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="O4" s="27"/>
+      <c r="Q4" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="S4" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="T4" s="27"/>
+      <c r="V4" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="X4" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y4" s="27"/>
+    </row>
+    <row r="5" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="C5" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="L5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="N5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="S5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="T5" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="V5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="X5" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="Y5" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="57">
+    </row>
+    <row r="6" spans="2:25" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="I6" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="J6" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q6" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="S6" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="T6" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="V6" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="X6" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y6" s="39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B7" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16"/>
+      <c r="W7" s="16"/>
+      <c r="X7" s="16"/>
+      <c r="Y7" s="43"/>
+    </row>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B8" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="8">
+        <f>'Series A'!C8</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="40"/>
+      <c r="E8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="N8" s="40"/>
+      <c r="O8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="S8" s="40"/>
+      <c r="T8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="X8" s="2">
+        <f>C8+E8+G8+J8+L8+O8+Q8+T8+V8</f>
+        <v>3600000</v>
+      </c>
+      <c r="Y8" s="50">
+        <f ca="1">X8/$X$22</f>
+        <v>0.14266248781820867</v>
+      </c>
+    </row>
+    <row r="9" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B9" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="8">
+        <f>'Series A'!C9</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="40"/>
+      <c r="E9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="N9" s="40"/>
+      <c r="O9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="S9" s="40"/>
+      <c r="T9" s="2"/>
+      <c r="V9" s="2"/>
+      <c r="X9" s="2">
+        <f>C9+E9+G9+J9+L9+O9+Q9+T9+V9</f>
+        <v>3600000</v>
+      </c>
+      <c r="Y9" s="50">
+        <f ca="1">X9/$X$22</f>
+        <v>0.14266248781820867</v>
+      </c>
+    </row>
+    <row r="10" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B10" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="8">
+        <f>'Series A'!C10</f>
+        <v>1429687</v>
+      </c>
+      <c r="D10" s="40"/>
+      <c r="E10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="I10" s="40"/>
+      <c r="J10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="N10" s="40"/>
+      <c r="O10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="S10" s="40"/>
+      <c r="T10" s="2"/>
+      <c r="V10" s="2"/>
+      <c r="X10" s="2">
+        <f>C10+E10+G10+J10+L10+O10+Q10+T10+V10</f>
+        <v>1429687</v>
+      </c>
+      <c r="Y10" s="50">
+        <f ca="1">X10/$X$22</f>
+        <v>5.6656306728153145E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B11" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="8">
+        <f>'Series A'!C11</f>
+        <v>1045471</v>
+      </c>
+      <c r="D11" s="40"/>
+      <c r="E11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="N11" s="40"/>
+      <c r="O11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="S11" s="40"/>
+      <c r="T11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="X11" s="2">
+        <f>C11+E11+G11+J11+L11+O11+Q11+T11+V11</f>
+        <v>1045471</v>
+      </c>
+      <c r="Y11" s="50">
+        <f ca="1">X11/$X$22</f>
+        <v>4.143041494494179E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B12" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="8">
+        <f>'Series A'!C12</f>
+        <v>65105</v>
+      </c>
+      <c r="D12" s="40"/>
+      <c r="E12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="N12" s="40"/>
+      <c r="O12" s="2"/>
+      <c r="Q12" s="2">
+        <f ca="1">'Series A'!Q13</f>
+        <v>1867629</v>
+      </c>
+      <c r="S12" s="40"/>
+      <c r="T12" s="2"/>
+      <c r="V12" s="2"/>
+      <c r="X12" s="2">
+        <f ca="1">C12+E12+G12+J12+L12+O12+Q12+T12+V12</f>
+        <v>1932734</v>
+      </c>
+      <c r="Y12" s="50">
+        <f ca="1">X12/$X$22</f>
+        <v>7.659128909189937E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="19"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="N13" s="40"/>
+      <c r="O13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="2"/>
+      <c r="V13" s="2">
+        <f ca="1">IFERROR(ROUND(X22*C34,0),0)</f>
+        <v>1766407</v>
+      </c>
+      <c r="X13" s="2">
+        <f ca="1">C13+E13+G13+J13+L13+O13+Q13+T13+V13</f>
+        <v>1766407</v>
+      </c>
+      <c r="Y13" s="50">
+        <f ca="1">X13/$X$22</f>
+        <v>7.0000004755416262E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B14" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="51">
+        <f>SUM(C8:C13)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D14" s="40">
+        <f>SUM(D8:D13)</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <f>SUM(E8:E13)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="51">
+        <f>SUM(G8:G13)</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="40"/>
+      <c r="J14" s="2">
+        <f>SUM(J8:J13)</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="51">
+        <f>SUM(L8:L13)</f>
+        <v>0</v>
+      </c>
+      <c r="N14" s="40"/>
+      <c r="O14" s="2">
+        <f>SUM(O8:O13)</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="51">
+        <f ca="1">SUM(Q8:Q13)</f>
+        <v>1867629</v>
+      </c>
+      <c r="S14" s="40"/>
+      <c r="T14" s="2">
+        <f>SUM(T8:T13)</f>
+        <v>0</v>
+      </c>
+      <c r="V14" s="51">
+        <f ca="1">SUM(V8:V13)</f>
+        <v>1766407</v>
+      </c>
+      <c r="X14" s="51">
+        <f ca="1">SUM(X8:X13)</f>
+        <v>13374299</v>
+      </c>
+      <c r="Y14" s="52">
+        <f ca="1">X14/$X$22</f>
+        <v>0.53000299115682792</v>
+      </c>
+    </row>
+    <row r="15" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B15" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="N15" s="40"/>
+      <c r="O15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="S15" s="40"/>
+      <c r="T15" s="2"/>
+      <c r="V15" s="2"/>
+      <c r="X15" s="2"/>
+      <c r="Y15" s="50"/>
+    </row>
+    <row r="16" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B16" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="57">
+        <f>'Series A'!D16</f>
+        <v>8000000</v>
+      </c>
+      <c r="E16" s="8">
+        <f ca="1">'Series A'!E16</f>
+        <v>2311471</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="N16" s="57">
+        <f>'Series A'!N16</f>
+        <v>5000000</v>
+      </c>
+      <c r="O16" s="8">
+        <f ca="1">'Series A'!O16</f>
+        <v>1203891</v>
+      </c>
+      <c r="Q16" s="2"/>
+      <c r="S16" s="40">
+        <f>($S$22-$S$20)*(N16/$N$22)</f>
+        <v>3750000</v>
+      </c>
+      <c r="T16" s="2">
+        <f ca="1">IFERROR(ROUND(S16/$T$24,0),0)</f>
+        <v>525718</v>
+      </c>
+      <c r="V16" s="2"/>
+      <c r="X16" s="2">
+        <f ca="1">E16+C16+J16+O16+T16</f>
+        <v>4041080</v>
+      </c>
+      <c r="Y16" s="50">
+        <f ca="1">X16/$X$22</f>
+        <v>0.16014181285344631</v>
+      </c>
+    </row>
+    <row r="17" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B17" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="N17" s="57">
+        <f>'Series A'!N17</f>
+        <v>12000000</v>
+      </c>
+      <c r="O17" s="8">
+        <f ca="1">'Series A'!O17</f>
+        <v>2889338</v>
+      </c>
+      <c r="Q17" s="2"/>
+      <c r="S17" s="40">
+        <f>($S$22-$S$20)*(N17/$N$22)</f>
+        <v>9000000</v>
+      </c>
+      <c r="T17" s="2">
+        <f ca="1">IFERROR(ROUND(S17/$T$24,0),0)</f>
+        <v>1261724</v>
+      </c>
+      <c r="V17" s="2"/>
+      <c r="X17" s="2">
+        <f ca="1">E17+C17+J17+O17+T17</f>
+        <v>4151062</v>
+      </c>
+      <c r="Y17" s="50">
+        <f ca="1">X17/$X$22</f>
+        <v>0.16450023111323026</v>
+      </c>
+    </row>
+    <row r="18" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B18" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="N18" s="57">
+        <f>'Series A'!N18</f>
+        <v>3000000</v>
+      </c>
+      <c r="O18" s="8">
+        <f ca="1">'Series A'!O18</f>
+        <v>722335</v>
+      </c>
+      <c r="Q18" s="2"/>
+      <c r="S18" s="40">
+        <f>($S$22-$S$20)*(N18/$N$22)</f>
+        <v>2250000</v>
+      </c>
+      <c r="T18" s="2">
+        <f ca="1">IFERROR(ROUND(S18/$T$24,0),0)</f>
+        <v>315431</v>
+      </c>
+      <c r="V18" s="2"/>
+      <c r="X18" s="2">
+        <f ca="1">E18+C18+J18+O18+T18</f>
+        <v>1037766</v>
+      </c>
+      <c r="Y18" s="50">
+        <f ca="1">X18/$X$22</f>
+        <v>4.1125077592541984E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B19" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="57">
+        <f>'Series A'!D19</f>
+        <v>1825000</v>
+      </c>
+      <c r="E19" s="8">
+        <f ca="1">'Series A'!E19</f>
+        <v>527304</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="N19" s="40"/>
+      <c r="O19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="S19" s="40"/>
+      <c r="T19" s="2"/>
+      <c r="V19" s="2"/>
+      <c r="X19" s="2">
+        <f ca="1">E19+C19+J19+O19+T19</f>
+        <v>527304</v>
+      </c>
+      <c r="Y19" s="50">
+        <f ca="1">X19/$X$22</f>
+        <v>2.0896250132359087E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B20" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="I20" s="40"/>
+      <c r="J20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="N20" s="40"/>
+      <c r="O20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="S20" s="63">
+        <v>15000000</v>
+      </c>
+      <c r="T20" s="2">
+        <f ca="1">IFERROR(ROUND(S20/$T$24,0),0)</f>
+        <v>2102873</v>
+      </c>
+      <c r="V20" s="2"/>
+      <c r="X20" s="2">
+        <f ca="1">E20+C20+J20+O20+T20</f>
+        <v>2102873</v>
+      </c>
+      <c r="Y20" s="50">
+        <f ca="1">X20/$X$22</f>
+        <v>8.3333637151594434E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B21" s="19"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="S21" s="40"/>
+      <c r="T21" s="2"/>
+      <c r="V21" s="2"/>
+      <c r="X21" s="2"/>
+      <c r="Y21" s="50"/>
+    </row>
+    <row r="22" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B22" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="53">
+        <f>C14+SUM(C16:C20)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D22" s="61">
+        <f>SUM(D8:D20)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E22" s="53">
+        <f ca="1">SUM(E8:E20)</f>
+        <v>2838775</v>
+      </c>
+      <c r="G22" s="51">
+        <f>G13</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="61">
+        <f>SUM(I16:I21)</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="53">
+        <f>SUM(J16:J21)</f>
+        <v>0</v>
+      </c>
+      <c r="L22" s="51">
+        <f>L13</f>
+        <v>0</v>
+      </c>
+      <c r="N22" s="61">
+        <f>SUM(N16:N20)</f>
+        <v>20000000</v>
+      </c>
+      <c r="O22" s="53">
+        <f ca="1">SUM(O16:O20)</f>
+        <v>4815564</v>
+      </c>
+      <c r="Q22" s="51">
+        <f ca="1">Q12</f>
+        <v>1867629</v>
+      </c>
+      <c r="S22" s="61">
+        <f>C31</f>
+        <v>30000000</v>
+      </c>
+      <c r="T22" s="53">
+        <f ca="1">SUM(T16:T21)</f>
+        <v>4205746</v>
+      </c>
+      <c r="V22" s="51">
+        <f ca="1">V13</f>
+        <v>1766407</v>
+      </c>
+      <c r="X22" s="53">
+        <f ca="1">SUM(X16:X21)+X14</f>
+        <v>25234384</v>
+      </c>
+      <c r="Y22" s="55">
+        <f ca="1">SUM(Y16:Y20)+Y14</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:25" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="19"/>
+      <c r="Y23" s="21"/>
+    </row>
+    <row r="24" spans="2:25" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" s="14">
+        <f ca="1">'Series A'!E23</f>
+        <v>3.4609999999999999</v>
+      </c>
+      <c r="J24" s="14">
+        <f ca="1">'Series A'!E23</f>
+        <v>3.4609999999999999</v>
+      </c>
+      <c r="O24" s="14">
+        <f ca="1">'Series A'!O23</f>
+        <v>4.1532</v>
+      </c>
+      <c r="T24" s="62">
+        <f ca="1">IFERROR(ROUND(T25/(Q22+O22+L22+J22+G22+V13+E22+C22),4),0)</f>
+        <v>7.1330999999999998</v>
+      </c>
+      <c r="Y24" s="21"/>
+    </row>
+    <row r="25" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B25" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E25" s="15">
+        <f>'Series A'!E25</f>
         <v>50000000</v>
+      </c>
+      <c r="J25" s="15">
+        <f>'Series A'!E25</f>
+        <v>50000000</v>
+      </c>
+      <c r="O25" s="15">
+        <f>'Series A'!O24</f>
+        <v>60000000</v>
+      </c>
+      <c r="T25" s="15">
+        <f>T26-S22</f>
+        <v>150000000</v>
+      </c>
+      <c r="Y25" s="21"/>
+    </row>
+    <row r="26" spans="2:25" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="42" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="18">
+        <f>'Series A'!E25</f>
+        <v>50000000</v>
+      </c>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="18">
+        <f>J25+I22</f>
+        <v>50000000</v>
+      </c>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="18">
+        <f>O25+N22</f>
+        <v>80000000</v>
+      </c>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="17"/>
+      <c r="R26" s="17"/>
+      <c r="S26" s="17"/>
+      <c r="T26" s="18">
+        <f>C31/C32</f>
+        <v>180000000</v>
+      </c>
+      <c r="U26" s="17"/>
+      <c r="V26" s="17"/>
+      <c r="W26" s="17"/>
+      <c r="X26" s="17"/>
+      <c r="Y26" s="22"/>
+    </row>
+    <row r="28" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" s="1">
+        <f>T25/O26-1</f>
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="31" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="63">
+        <v>30000000</v>
+      </c>
+    </row>
+    <row r="32" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>78</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>92</v>
+      </c>
+      <c r="C33" s="1">
+        <f>S20/S22</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>103</v>
+      </c>
+      <c r="C34" s="10">
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>